<commit_message>
All working for Office
</commit_message>
<xml_diff>
--- a/thaco/color/Office-1_color.xlsx
+++ b/thaco/color/Office-1_color.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adity/Documents/GitHub/gitlocal/thaco/color/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3544D12F-1D86-D441-AEA4-106B5843F08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E6CBC2-893A-A542-A2B4-91669771821F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="39640" yWindow="500" windowWidth="38100" windowHeight="20800" tabRatio="761" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6736,7 +6736,6 @@
     <xf numFmtId="164" fontId="66" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="28" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6976,6 +6975,7 @@
     <xf numFmtId="164" fontId="42" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="1991-" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -7742,88 +7742,88 @@
       <c r="CD2" s="296"/>
     </row>
     <row r="3" spans="1:87" s="14" customFormat="1" ht="24" customHeight="1" outlineLevel="1">
-      <c r="A3" s="366"/>
-      <c r="B3" s="363"/>
-      <c r="C3" s="363"/>
-      <c r="D3" s="363"/>
-      <c r="E3" s="363"/>
-      <c r="F3" s="363"/>
-      <c r="G3" s="363"/>
-      <c r="H3" s="363"/>
-      <c r="I3" s="363"/>
-      <c r="J3" s="363"/>
-      <c r="K3" s="363"/>
-      <c r="L3" s="363"/>
-      <c r="M3" s="363"/>
-      <c r="N3" s="363"/>
-      <c r="O3" s="363"/>
-      <c r="P3" s="363"/>
-      <c r="Q3" s="363"/>
-      <c r="R3" s="363"/>
-      <c r="S3" s="363"/>
-      <c r="T3" s="363"/>
-      <c r="U3" s="363"/>
-      <c r="V3" s="363"/>
-      <c r="W3" s="363"/>
-      <c r="X3" s="363"/>
-      <c r="Y3" s="363"/>
-      <c r="Z3" s="363"/>
-      <c r="AA3" s="363"/>
-      <c r="AB3" s="363"/>
-      <c r="AC3" s="363"/>
-      <c r="AD3" s="363"/>
-      <c r="AE3" s="363"/>
-      <c r="AF3" s="363"/>
-      <c r="AG3" s="363"/>
-      <c r="AH3" s="363"/>
-      <c r="AI3" s="363"/>
-      <c r="AJ3" s="363"/>
-      <c r="AK3" s="363"/>
-      <c r="AL3" s="363"/>
-      <c r="AM3" s="363"/>
-      <c r="AN3" s="363"/>
-      <c r="AO3" s="363"/>
-      <c r="AP3" s="363"/>
-      <c r="AQ3" s="363"/>
-      <c r="AR3" s="363"/>
-      <c r="AS3" s="363"/>
-      <c r="AT3" s="363"/>
-      <c r="AU3" s="363"/>
-      <c r="AV3" s="363"/>
-      <c r="AW3" s="363"/>
-      <c r="AX3" s="363"/>
-      <c r="AY3" s="363"/>
-      <c r="AZ3" s="363"/>
-      <c r="BA3" s="363"/>
-      <c r="BB3" s="363"/>
-      <c r="BC3" s="363"/>
-      <c r="BD3" s="363"/>
-      <c r="BE3" s="363"/>
-      <c r="BF3" s="363"/>
-      <c r="BG3" s="363"/>
-      <c r="BH3" s="363"/>
-      <c r="BI3" s="363"/>
-      <c r="BJ3" s="363"/>
-      <c r="BK3" s="363"/>
-      <c r="BL3" s="363"/>
-      <c r="BM3" s="363"/>
-      <c r="BN3" s="363"/>
-      <c r="BO3" s="363"/>
-      <c r="BP3" s="363"/>
-      <c r="BQ3" s="363"/>
-      <c r="BR3" s="363"/>
-      <c r="BS3" s="363"/>
-      <c r="BT3" s="363"/>
-      <c r="BU3" s="363"/>
+      <c r="A3" s="365"/>
+      <c r="B3" s="362"/>
+      <c r="C3" s="362"/>
+      <c r="D3" s="362"/>
+      <c r="E3" s="362"/>
+      <c r="F3" s="362"/>
+      <c r="G3" s="362"/>
+      <c r="H3" s="362"/>
+      <c r="I3" s="362"/>
+      <c r="J3" s="362"/>
+      <c r="K3" s="362"/>
+      <c r="L3" s="362"/>
+      <c r="M3" s="362"/>
+      <c r="N3" s="362"/>
+      <c r="O3" s="362"/>
+      <c r="P3" s="362"/>
+      <c r="Q3" s="362"/>
+      <c r="R3" s="362"/>
+      <c r="S3" s="362"/>
+      <c r="T3" s="362"/>
+      <c r="U3" s="362"/>
+      <c r="V3" s="362"/>
+      <c r="W3" s="362"/>
+      <c r="X3" s="362"/>
+      <c r="Y3" s="362"/>
+      <c r="Z3" s="362"/>
+      <c r="AA3" s="362"/>
+      <c r="AB3" s="362"/>
+      <c r="AC3" s="362"/>
+      <c r="AD3" s="362"/>
+      <c r="AE3" s="362"/>
+      <c r="AF3" s="362"/>
+      <c r="AG3" s="362"/>
+      <c r="AH3" s="362"/>
+      <c r="AI3" s="362"/>
+      <c r="AJ3" s="362"/>
+      <c r="AK3" s="362"/>
+      <c r="AL3" s="362"/>
+      <c r="AM3" s="362"/>
+      <c r="AN3" s="362"/>
+      <c r="AO3" s="362"/>
+      <c r="AP3" s="362"/>
+      <c r="AQ3" s="362"/>
+      <c r="AR3" s="362"/>
+      <c r="AS3" s="362"/>
+      <c r="AT3" s="362"/>
+      <c r="AU3" s="362"/>
+      <c r="AV3" s="362"/>
+      <c r="AW3" s="362"/>
+      <c r="AX3" s="362"/>
+      <c r="AY3" s="362"/>
+      <c r="AZ3" s="362"/>
+      <c r="BA3" s="362"/>
+      <c r="BB3" s="362"/>
+      <c r="BC3" s="362"/>
+      <c r="BD3" s="362"/>
+      <c r="BE3" s="362"/>
+      <c r="BF3" s="362"/>
+      <c r="BG3" s="362"/>
+      <c r="BH3" s="362"/>
+      <c r="BI3" s="362"/>
+      <c r="BJ3" s="362"/>
+      <c r="BK3" s="362"/>
+      <c r="BL3" s="362"/>
+      <c r="BM3" s="362"/>
+      <c r="BN3" s="362"/>
+      <c r="BO3" s="362"/>
+      <c r="BP3" s="362"/>
+      <c r="BQ3" s="362"/>
+      <c r="BR3" s="362"/>
+      <c r="BS3" s="362"/>
+      <c r="BT3" s="362"/>
+      <c r="BU3" s="362"/>
       <c r="BV3" s="298"/>
-      <c r="BW3" s="362" t="s">
+      <c r="BW3" s="361" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="363"/>
-      <c r="BY3" s="363"/>
-      <c r="BZ3" s="363"/>
-      <c r="CA3" s="363"/>
-      <c r="CB3" s="363"/>
+      <c r="BX3" s="362"/>
+      <c r="BY3" s="362"/>
+      <c r="BZ3" s="362"/>
+      <c r="CA3" s="362"/>
+      <c r="CB3" s="362"/>
       <c r="CC3" s="300"/>
       <c r="CD3" s="300"/>
     </row>
@@ -7901,12 +7901,12 @@
       <c r="BT4" s="301"/>
       <c r="BU4" s="301"/>
       <c r="BV4" s="301"/>
-      <c r="BW4" s="363"/>
-      <c r="BX4" s="363"/>
-      <c r="BY4" s="363"/>
-      <c r="BZ4" s="363"/>
-      <c r="CA4" s="363"/>
-      <c r="CB4" s="363"/>
+      <c r="BW4" s="362"/>
+      <c r="BX4" s="362"/>
+      <c r="BY4" s="362"/>
+      <c r="BZ4" s="362"/>
+      <c r="CA4" s="362"/>
+      <c r="CB4" s="362"/>
       <c r="CC4" s="300"/>
       <c r="CD4" s="300"/>
     </row>
@@ -7984,12 +7984,12 @@
       <c r="BT5" s="301"/>
       <c r="BU5" s="301"/>
       <c r="BV5" s="301"/>
-      <c r="BW5" s="363"/>
-      <c r="BX5" s="363"/>
-      <c r="BY5" s="363"/>
-      <c r="BZ5" s="363"/>
-      <c r="CA5" s="363"/>
-      <c r="CB5" s="363"/>
+      <c r="BW5" s="362"/>
+      <c r="BX5" s="362"/>
+      <c r="BY5" s="362"/>
+      <c r="BZ5" s="362"/>
+      <c r="CA5" s="362"/>
+      <c r="CB5" s="362"/>
       <c r="CC5" s="300"/>
       <c r="CD5" s="300"/>
     </row>
@@ -8065,12 +8065,12 @@
       <c r="BT6" s="303"/>
       <c r="BU6" s="303"/>
       <c r="BV6" s="303"/>
-      <c r="BW6" s="363"/>
-      <c r="BX6" s="363"/>
-      <c r="BY6" s="363"/>
-      <c r="BZ6" s="363"/>
-      <c r="CA6" s="363"/>
-      <c r="CB6" s="363"/>
+      <c r="BW6" s="362"/>
+      <c r="BX6" s="362"/>
+      <c r="BY6" s="362"/>
+      <c r="BZ6" s="362"/>
+      <c r="CA6" s="362"/>
+      <c r="CB6" s="362"/>
       <c r="CC6" s="300"/>
       <c r="CD6" s="300"/>
     </row>
@@ -8210,356 +8210,356 @@
       </c>
     </row>
     <row r="8" spans="1:87" s="306" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A8" s="334" t="s">
+      <c r="A8" s="333" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="368" t="s">
+      <c r="B8" s="367" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="346" t="s">
+      <c r="C8" s="345" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="350" t="s">
+      <c r="D8" s="349" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="350" t="s">
+      <c r="E8" s="349" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="346" t="s">
+      <c r="F8" s="345" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="369" t="s">
+      <c r="G8" s="368" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="355" t="s">
+      <c r="H8" s="354" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="355" t="s">
+      <c r="I8" s="354" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="355" t="s">
+      <c r="J8" s="354" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="356" t="s">
+      <c r="K8" s="355" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="357"/>
-      <c r="M8" s="357"/>
-      <c r="N8" s="357"/>
-      <c r="O8" s="357"/>
-      <c r="P8" s="357"/>
-      <c r="Q8" s="357"/>
-      <c r="R8" s="357"/>
-      <c r="S8" s="357"/>
-      <c r="T8" s="357"/>
-      <c r="U8" s="357"/>
-      <c r="V8" s="357"/>
-      <c r="W8" s="357"/>
-      <c r="X8" s="357"/>
-      <c r="Y8" s="361" t="s">
+      <c r="L8" s="356"/>
+      <c r="M8" s="356"/>
+      <c r="N8" s="356"/>
+      <c r="O8" s="356"/>
+      <c r="P8" s="356"/>
+      <c r="Q8" s="356"/>
+      <c r="R8" s="356"/>
+      <c r="S8" s="356"/>
+      <c r="T8" s="356"/>
+      <c r="U8" s="356"/>
+      <c r="V8" s="356"/>
+      <c r="W8" s="356"/>
+      <c r="X8" s="356"/>
+      <c r="Y8" s="360" t="s">
         <v>15</v>
       </c>
-      <c r="Z8" s="357"/>
-      <c r="AA8" s="357"/>
-      <c r="AB8" s="357"/>
-      <c r="AC8" s="357"/>
-      <c r="AD8" s="357"/>
-      <c r="AE8" s="357"/>
-      <c r="AF8" s="357"/>
-      <c r="AG8" s="357"/>
-      <c r="AH8" s="357"/>
-      <c r="AI8" s="357"/>
-      <c r="AJ8" s="357"/>
-      <c r="AK8" s="357"/>
-      <c r="AL8" s="357"/>
-      <c r="AM8" s="357"/>
-      <c r="AN8" s="357"/>
-      <c r="AO8" s="359"/>
-      <c r="AP8" s="355" t="s">
+      <c r="Z8" s="356"/>
+      <c r="AA8" s="356"/>
+      <c r="AB8" s="356"/>
+      <c r="AC8" s="356"/>
+      <c r="AD8" s="356"/>
+      <c r="AE8" s="356"/>
+      <c r="AF8" s="356"/>
+      <c r="AG8" s="356"/>
+      <c r="AH8" s="356"/>
+      <c r="AI8" s="356"/>
+      <c r="AJ8" s="356"/>
+      <c r="AK8" s="356"/>
+      <c r="AL8" s="356"/>
+      <c r="AM8" s="356"/>
+      <c r="AN8" s="356"/>
+      <c r="AO8" s="358"/>
+      <c r="AP8" s="354" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="355" t="s">
+      <c r="AQ8" s="354" t="s">
         <v>17</v>
       </c>
-      <c r="AR8" s="355" t="s">
+      <c r="AR8" s="354" t="s">
         <v>18</v>
       </c>
-      <c r="AS8" s="355" t="s">
+      <c r="AS8" s="354" t="s">
         <v>19</v>
       </c>
-      <c r="AT8" s="355" t="s">
+      <c r="AT8" s="354" t="s">
         <v>20</v>
       </c>
-      <c r="AU8" s="355" t="s">
+      <c r="AU8" s="354" t="s">
         <v>21</v>
       </c>
-      <c r="AV8" s="346" t="s">
+      <c r="AV8" s="345" t="s">
         <v>22</v>
       </c>
-      <c r="AW8" s="360" t="s">
+      <c r="AW8" s="359" t="s">
         <v>23</v>
       </c>
-      <c r="AX8" s="360" t="s">
+      <c r="AX8" s="359" t="s">
         <v>24</v>
       </c>
-      <c r="AY8" s="358" t="s">
+      <c r="AY8" s="357" t="s">
         <v>25</v>
       </c>
-      <c r="AZ8" s="357"/>
-      <c r="BA8" s="357"/>
-      <c r="BB8" s="357"/>
-      <c r="BC8" s="357"/>
-      <c r="BD8" s="357"/>
-      <c r="BE8" s="357"/>
-      <c r="BF8" s="357"/>
-      <c r="BG8" s="357"/>
-      <c r="BH8" s="357"/>
-      <c r="BI8" s="357"/>
-      <c r="BJ8" s="357"/>
-      <c r="BK8" s="357"/>
-      <c r="BL8" s="357"/>
-      <c r="BM8" s="357"/>
-      <c r="BN8" s="357"/>
-      <c r="BO8" s="357"/>
-      <c r="BP8" s="357"/>
-      <c r="BQ8" s="359"/>
-      <c r="BR8" s="377" t="s">
+      <c r="AZ8" s="356"/>
+      <c r="BA8" s="356"/>
+      <c r="BB8" s="356"/>
+      <c r="BC8" s="356"/>
+      <c r="BD8" s="356"/>
+      <c r="BE8" s="356"/>
+      <c r="BF8" s="356"/>
+      <c r="BG8" s="356"/>
+      <c r="BH8" s="356"/>
+      <c r="BI8" s="356"/>
+      <c r="BJ8" s="356"/>
+      <c r="BK8" s="356"/>
+      <c r="BL8" s="356"/>
+      <c r="BM8" s="356"/>
+      <c r="BN8" s="356"/>
+      <c r="BO8" s="356"/>
+      <c r="BP8" s="356"/>
+      <c r="BQ8" s="358"/>
+      <c r="BR8" s="376" t="s">
         <v>26</v>
       </c>
-      <c r="BS8" s="374"/>
-      <c r="BT8" s="346" t="s">
+      <c r="BS8" s="373"/>
+      <c r="BT8" s="345" t="s">
         <v>27</v>
       </c>
-      <c r="BU8" s="370" t="s">
+      <c r="BU8" s="369" t="s">
         <v>28</v>
       </c>
       <c r="BV8" s="22"/>
-      <c r="BW8" s="347" t="s">
+      <c r="BW8" s="346" t="s">
         <v>29</v>
       </c>
-      <c r="BX8" s="337" t="s">
+      <c r="BX8" s="336" t="s">
         <v>30</v>
       </c>
-      <c r="BY8" s="338"/>
-      <c r="BZ8" s="338"/>
-      <c r="CA8" s="339"/>
-      <c r="CB8" s="378" t="s">
+      <c r="BY8" s="337"/>
+      <c r="BZ8" s="337"/>
+      <c r="CA8" s="338"/>
+      <c r="CB8" s="377" t="s">
         <v>31</v>
       </c>
-      <c r="CC8" s="364" t="s">
+      <c r="CC8" s="363" t="s">
         <v>32</v>
       </c>
-      <c r="CD8" s="364" t="s">
+      <c r="CD8" s="363" t="s">
         <v>33</v>
       </c>
       <c r="CH8" s="241"/>
       <c r="CI8" s="241"/>
     </row>
     <row r="9" spans="1:87" s="306" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A9" s="335"/>
-      <c r="B9" s="332"/>
-      <c r="C9" s="332"/>
-      <c r="D9" s="332"/>
-      <c r="E9" s="332"/>
-      <c r="F9" s="332"/>
-      <c r="G9" s="332"/>
-      <c r="H9" s="335"/>
-      <c r="I9" s="335"/>
-      <c r="J9" s="335"/>
-      <c r="K9" s="353" t="s">
+      <c r="A9" s="334"/>
+      <c r="B9" s="331"/>
+      <c r="C9" s="331"/>
+      <c r="D9" s="331"/>
+      <c r="E9" s="331"/>
+      <c r="F9" s="331"/>
+      <c r="G9" s="331"/>
+      <c r="H9" s="334"/>
+      <c r="I9" s="334"/>
+      <c r="J9" s="334"/>
+      <c r="K9" s="352" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="353" t="s">
+      <c r="L9" s="352" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="353" t="s">
+      <c r="M9" s="352" t="s">
         <v>36</v>
       </c>
-      <c r="N9" s="353" t="s">
+      <c r="N9" s="352" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="353" t="s">
+      <c r="O9" s="352" t="s">
         <v>38</v>
       </c>
-      <c r="P9" s="353" t="s">
+      <c r="P9" s="352" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="353" t="s">
+      <c r="Q9" s="352" t="s">
         <v>40</v>
       </c>
-      <c r="R9" s="353" t="s">
+      <c r="R9" s="352" t="s">
         <v>41</v>
       </c>
-      <c r="S9" s="353" t="s">
+      <c r="S9" s="352" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="353" t="s">
+      <c r="T9" s="352" t="s">
         <v>43</v>
       </c>
-      <c r="U9" s="353" t="s">
+      <c r="U9" s="352" t="s">
         <v>44</v>
       </c>
-      <c r="V9" s="373" t="s">
+      <c r="V9" s="372" t="s">
         <v>45</v>
       </c>
-      <c r="W9" s="374"/>
-      <c r="X9" s="353" t="s">
+      <c r="W9" s="373"/>
+      <c r="X9" s="352" t="s">
         <v>46</v>
       </c>
-      <c r="Y9" s="331" t="s">
+      <c r="Y9" s="330" t="s">
         <v>154</v>
       </c>
-      <c r="Z9" s="331" t="s">
+      <c r="Z9" s="330" t="s">
         <v>48</v>
       </c>
-      <c r="AA9" s="331" t="s">
+      <c r="AA9" s="330" t="s">
         <v>49</v>
       </c>
-      <c r="AB9" s="331" t="s">
+      <c r="AB9" s="330" t="s">
         <v>50</v>
       </c>
-      <c r="AC9" s="331" t="s">
+      <c r="AC9" s="330" t="s">
         <v>51</v>
       </c>
-      <c r="AD9" s="331" t="s">
+      <c r="AD9" s="330" t="s">
         <v>52</v>
       </c>
-      <c r="AE9" s="331" t="s">
+      <c r="AE9" s="330" t="s">
         <v>53</v>
       </c>
-      <c r="AF9" s="331" t="s">
+      <c r="AF9" s="330" t="s">
         <v>54</v>
       </c>
-      <c r="AG9" s="331" t="s">
+      <c r="AG9" s="330" t="s">
         <v>55</v>
       </c>
-      <c r="AH9" s="331" t="s">
+      <c r="AH9" s="330" t="s">
         <v>56</v>
       </c>
-      <c r="AI9" s="331" t="s">
+      <c r="AI9" s="330" t="s">
         <v>57</v>
       </c>
-      <c r="AJ9" s="331" t="s">
+      <c r="AJ9" s="330" t="s">
         <v>58</v>
       </c>
-      <c r="AK9" s="370" t="s">
+      <c r="AK9" s="369" t="s">
         <v>59</v>
       </c>
-      <c r="AL9" s="346" t="s">
+      <c r="AL9" s="345" t="s">
         <v>60</v>
       </c>
-      <c r="AM9" s="331" t="s">
+      <c r="AM9" s="330" t="s">
         <v>61</v>
       </c>
-      <c r="AN9" s="346" t="s">
+      <c r="AN9" s="345" t="s">
         <v>62</v>
       </c>
-      <c r="AO9" s="346" t="s">
+      <c r="AO9" s="345" t="s">
         <v>63</v>
       </c>
-      <c r="AP9" s="335"/>
-      <c r="AQ9" s="335"/>
-      <c r="AR9" s="335"/>
-      <c r="AS9" s="335"/>
-      <c r="AT9" s="335"/>
-      <c r="AU9" s="335"/>
-      <c r="AV9" s="332"/>
-      <c r="AW9" s="335"/>
-      <c r="AX9" s="335"/>
-      <c r="AY9" s="380" t="s">
+      <c r="AP9" s="334"/>
+      <c r="AQ9" s="334"/>
+      <c r="AR9" s="334"/>
+      <c r="AS9" s="334"/>
+      <c r="AT9" s="334"/>
+      <c r="AU9" s="334"/>
+      <c r="AV9" s="331"/>
+      <c r="AW9" s="334"/>
+      <c r="AX9" s="334"/>
+      <c r="AY9" s="379" t="s">
         <v>25</v>
       </c>
-      <c r="AZ9" s="381"/>
-      <c r="BA9" s="381"/>
-      <c r="BB9" s="381"/>
-      <c r="BC9" s="381"/>
-      <c r="BD9" s="381"/>
-      <c r="BE9" s="381"/>
-      <c r="BF9" s="381"/>
-      <c r="BG9" s="381"/>
-      <c r="BH9" s="381"/>
-      <c r="BI9" s="381"/>
-      <c r="BJ9" s="381"/>
-      <c r="BK9" s="381"/>
-      <c r="BL9" s="382"/>
-      <c r="BM9" s="380" t="s">
+      <c r="AZ9" s="380"/>
+      <c r="BA9" s="380"/>
+      <c r="BB9" s="380"/>
+      <c r="BC9" s="380"/>
+      <c r="BD9" s="380"/>
+      <c r="BE9" s="380"/>
+      <c r="BF9" s="380"/>
+      <c r="BG9" s="380"/>
+      <c r="BH9" s="380"/>
+      <c r="BI9" s="380"/>
+      <c r="BJ9" s="380"/>
+      <c r="BK9" s="380"/>
+      <c r="BL9" s="381"/>
+      <c r="BM9" s="379" t="s">
         <v>64</v>
       </c>
-      <c r="BN9" s="381"/>
-      <c r="BO9" s="381"/>
-      <c r="BP9" s="381"/>
-      <c r="BQ9" s="382"/>
-      <c r="BR9" s="354" t="s">
+      <c r="BN9" s="380"/>
+      <c r="BO9" s="380"/>
+      <c r="BP9" s="380"/>
+      <c r="BQ9" s="381"/>
+      <c r="BR9" s="353" t="s">
         <v>65</v>
       </c>
-      <c r="BS9" s="354" t="s">
+      <c r="BS9" s="353" t="s">
         <v>66</v>
       </c>
-      <c r="BT9" s="332"/>
-      <c r="BU9" s="371"/>
+      <c r="BT9" s="331"/>
+      <c r="BU9" s="370"/>
       <c r="BV9" s="22"/>
-      <c r="BW9" s="348"/>
-      <c r="BX9" s="340"/>
-      <c r="BY9" s="341"/>
-      <c r="BZ9" s="341"/>
-      <c r="CA9" s="342"/>
-      <c r="CB9" s="332"/>
-      <c r="CC9" s="335"/>
-      <c r="CD9" s="335"/>
+      <c r="BW9" s="347"/>
+      <c r="BX9" s="339"/>
+      <c r="BY9" s="340"/>
+      <c r="BZ9" s="340"/>
+      <c r="CA9" s="341"/>
+      <c r="CB9" s="331"/>
+      <c r="CC9" s="334"/>
+      <c r="CD9" s="334"/>
       <c r="CH9" s="241"/>
       <c r="CI9" s="241"/>
     </row>
     <row r="10" spans="1:87" s="307" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A10" s="335"/>
-      <c r="B10" s="332"/>
-      <c r="C10" s="332"/>
-      <c r="D10" s="332"/>
-      <c r="E10" s="332"/>
-      <c r="F10" s="332"/>
-      <c r="G10" s="332"/>
-      <c r="H10" s="335"/>
-      <c r="I10" s="335"/>
-      <c r="J10" s="335"/>
-      <c r="K10" s="335"/>
-      <c r="L10" s="335"/>
-      <c r="M10" s="335"/>
-      <c r="N10" s="335"/>
-      <c r="O10" s="335"/>
-      <c r="P10" s="335"/>
-      <c r="Q10" s="335"/>
-      <c r="R10" s="335"/>
-      <c r="S10" s="335"/>
-      <c r="T10" s="335"/>
-      <c r="U10" s="335"/>
-      <c r="V10" s="375"/>
-      <c r="W10" s="376"/>
-      <c r="X10" s="335"/>
-      <c r="Y10" s="332"/>
-      <c r="Z10" s="332"/>
-      <c r="AA10" s="332"/>
-      <c r="AB10" s="332"/>
-      <c r="AC10" s="332"/>
-      <c r="AD10" s="332"/>
-      <c r="AE10" s="332"/>
-      <c r="AF10" s="332"/>
-      <c r="AG10" s="332"/>
-      <c r="AH10" s="332"/>
-      <c r="AI10" s="332"/>
-      <c r="AJ10" s="332"/>
-      <c r="AK10" s="371"/>
-      <c r="AL10" s="332"/>
-      <c r="AM10" s="332"/>
-      <c r="AN10" s="332"/>
-      <c r="AO10" s="332"/>
-      <c r="AP10" s="335"/>
-      <c r="AQ10" s="335"/>
-      <c r="AR10" s="335"/>
-      <c r="AS10" s="335"/>
-      <c r="AT10" s="335"/>
-      <c r="AU10" s="335"/>
-      <c r="AV10" s="332"/>
-      <c r="AW10" s="335"/>
-      <c r="AX10" s="335"/>
+      <c r="A10" s="334"/>
+      <c r="B10" s="331"/>
+      <c r="C10" s="331"/>
+      <c r="D10" s="331"/>
+      <c r="E10" s="331"/>
+      <c r="F10" s="331"/>
+      <c r="G10" s="331"/>
+      <c r="H10" s="334"/>
+      <c r="I10" s="334"/>
+      <c r="J10" s="334"/>
+      <c r="K10" s="334"/>
+      <c r="L10" s="334"/>
+      <c r="M10" s="334"/>
+      <c r="N10" s="334"/>
+      <c r="O10" s="334"/>
+      <c r="P10" s="334"/>
+      <c r="Q10" s="334"/>
+      <c r="R10" s="334"/>
+      <c r="S10" s="334"/>
+      <c r="T10" s="334"/>
+      <c r="U10" s="334"/>
+      <c r="V10" s="374"/>
+      <c r="W10" s="375"/>
+      <c r="X10" s="334"/>
+      <c r="Y10" s="331"/>
+      <c r="Z10" s="331"/>
+      <c r="AA10" s="331"/>
+      <c r="AB10" s="331"/>
+      <c r="AC10" s="331"/>
+      <c r="AD10" s="331"/>
+      <c r="AE10" s="331"/>
+      <c r="AF10" s="331"/>
+      <c r="AG10" s="331"/>
+      <c r="AH10" s="331"/>
+      <c r="AI10" s="331"/>
+      <c r="AJ10" s="331"/>
+      <c r="AK10" s="370"/>
+      <c r="AL10" s="331"/>
+      <c r="AM10" s="331"/>
+      <c r="AN10" s="331"/>
+      <c r="AO10" s="331"/>
+      <c r="AP10" s="334"/>
+      <c r="AQ10" s="334"/>
+      <c r="AR10" s="334"/>
+      <c r="AS10" s="334"/>
+      <c r="AT10" s="334"/>
+      <c r="AU10" s="334"/>
+      <c r="AV10" s="331"/>
+      <c r="AW10" s="334"/>
+      <c r="AX10" s="334"/>
       <c r="AY10" s="101" t="s">
         <v>67</v>
       </c>
@@ -8569,67 +8569,67 @@
       <c r="BA10" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="BB10" s="367" t="s">
+      <c r="BB10" s="366" t="s">
         <v>70</v>
       </c>
-      <c r="BC10" s="352" t="s">
+      <c r="BC10" s="351" t="s">
         <v>71</v>
       </c>
-      <c r="BD10" s="352" t="s">
+      <c r="BD10" s="351" t="s">
         <v>72</v>
       </c>
-      <c r="BE10" s="351" t="s">
+      <c r="BE10" s="350" t="s">
         <v>73</v>
       </c>
-      <c r="BF10" s="351" t="s">
+      <c r="BF10" s="350" t="s">
         <v>74</v>
       </c>
-      <c r="BG10" s="352" t="s">
+      <c r="BG10" s="351" t="s">
         <v>75</v>
       </c>
-      <c r="BH10" s="352" t="s">
+      <c r="BH10" s="351" t="s">
         <v>76</v>
       </c>
-      <c r="BI10" s="351" t="s">
+      <c r="BI10" s="350" t="s">
         <v>77</v>
       </c>
-      <c r="BJ10" s="351" t="s">
+      <c r="BJ10" s="350" t="s">
         <v>78</v>
       </c>
-      <c r="BK10" s="351" t="s">
+      <c r="BK10" s="350" t="s">
         <v>79</v>
       </c>
-      <c r="BL10" s="346" t="s">
+      <c r="BL10" s="345" t="s">
         <v>80</v>
       </c>
-      <c r="BM10" s="352" t="s">
+      <c r="BM10" s="351" t="s">
         <v>81</v>
       </c>
-      <c r="BN10" s="360" t="s">
+      <c r="BN10" s="359" t="s">
         <v>82</v>
       </c>
-      <c r="BO10" s="352" t="s">
+      <c r="BO10" s="351" t="s">
         <v>83</v>
       </c>
-      <c r="BP10" s="360" t="s">
+      <c r="BP10" s="359" t="s">
         <v>84</v>
       </c>
-      <c r="BQ10" s="360" t="s">
+      <c r="BQ10" s="359" t="s">
         <v>85</v>
       </c>
-      <c r="BR10" s="335"/>
-      <c r="BS10" s="335"/>
-      <c r="BT10" s="332"/>
-      <c r="BU10" s="371"/>
+      <c r="BR10" s="334"/>
+      <c r="BS10" s="334"/>
+      <c r="BT10" s="331"/>
+      <c r="BU10" s="370"/>
       <c r="BV10" s="22"/>
-      <c r="BW10" s="348"/>
-      <c r="BX10" s="343"/>
-      <c r="BY10" s="344"/>
-      <c r="BZ10" s="344"/>
-      <c r="CA10" s="345"/>
-      <c r="CB10" s="332"/>
-      <c r="CC10" s="335"/>
-      <c r="CD10" s="335"/>
+      <c r="BW10" s="347"/>
+      <c r="BX10" s="342"/>
+      <c r="BY10" s="343"/>
+      <c r="BZ10" s="343"/>
+      <c r="CA10" s="344"/>
+      <c r="CB10" s="331"/>
+      <c r="CC10" s="334"/>
+      <c r="CD10" s="334"/>
       <c r="CE10" s="321" t="s">
         <v>3</v>
       </c>
@@ -8637,60 +8637,60 @@
       <c r="CI10" s="241"/>
     </row>
     <row r="11" spans="1:87" s="307" customFormat="1" ht="38.25" customHeight="1">
-      <c r="A11" s="336"/>
-      <c r="B11" s="333"/>
-      <c r="C11" s="333"/>
-      <c r="D11" s="333"/>
-      <c r="E11" s="333"/>
-      <c r="F11" s="333"/>
-      <c r="G11" s="333"/>
-      <c r="H11" s="336"/>
-      <c r="I11" s="336"/>
-      <c r="J11" s="336"/>
-      <c r="K11" s="336"/>
-      <c r="L11" s="336"/>
-      <c r="M11" s="336"/>
-      <c r="N11" s="336"/>
-      <c r="O11" s="336"/>
-      <c r="P11" s="336"/>
-      <c r="Q11" s="336"/>
-      <c r="R11" s="336"/>
-      <c r="S11" s="336"/>
-      <c r="T11" s="336"/>
-      <c r="U11" s="336"/>
+      <c r="A11" s="335"/>
+      <c r="B11" s="332"/>
+      <c r="C11" s="332"/>
+      <c r="D11" s="332"/>
+      <c r="E11" s="332"/>
+      <c r="F11" s="332"/>
+      <c r="G11" s="332"/>
+      <c r="H11" s="335"/>
+      <c r="I11" s="335"/>
+      <c r="J11" s="335"/>
+      <c r="K11" s="335"/>
+      <c r="L11" s="335"/>
+      <c r="M11" s="335"/>
+      <c r="N11" s="335"/>
+      <c r="O11" s="335"/>
+      <c r="P11" s="335"/>
+      <c r="Q11" s="335"/>
+      <c r="R11" s="335"/>
+      <c r="S11" s="335"/>
+      <c r="T11" s="335"/>
+      <c r="U11" s="335"/>
       <c r="V11" s="269" t="s">
         <v>86</v>
       </c>
       <c r="W11" s="269" t="s">
         <v>87</v>
       </c>
-      <c r="X11" s="336"/>
-      <c r="Y11" s="333"/>
-      <c r="Z11" s="333"/>
-      <c r="AA11" s="333"/>
-      <c r="AB11" s="333"/>
-      <c r="AC11" s="333"/>
-      <c r="AD11" s="333"/>
-      <c r="AE11" s="333"/>
-      <c r="AF11" s="333"/>
-      <c r="AG11" s="333"/>
-      <c r="AH11" s="333"/>
-      <c r="AI11" s="333"/>
-      <c r="AJ11" s="333"/>
-      <c r="AK11" s="372"/>
-      <c r="AL11" s="333"/>
-      <c r="AM11" s="333"/>
-      <c r="AN11" s="333"/>
-      <c r="AO11" s="333"/>
-      <c r="AP11" s="336"/>
-      <c r="AQ11" s="336"/>
-      <c r="AR11" s="336"/>
-      <c r="AS11" s="336"/>
-      <c r="AT11" s="336"/>
-      <c r="AU11" s="336"/>
-      <c r="AV11" s="333"/>
-      <c r="AW11" s="336"/>
-      <c r="AX11" s="336"/>
+      <c r="X11" s="335"/>
+      <c r="Y11" s="332"/>
+      <c r="Z11" s="332"/>
+      <c r="AA11" s="332"/>
+      <c r="AB11" s="332"/>
+      <c r="AC11" s="332"/>
+      <c r="AD11" s="332"/>
+      <c r="AE11" s="332"/>
+      <c r="AF11" s="332"/>
+      <c r="AG11" s="332"/>
+      <c r="AH11" s="332"/>
+      <c r="AI11" s="332"/>
+      <c r="AJ11" s="332"/>
+      <c r="AK11" s="371"/>
+      <c r="AL11" s="332"/>
+      <c r="AM11" s="332"/>
+      <c r="AN11" s="332"/>
+      <c r="AO11" s="332"/>
+      <c r="AP11" s="335"/>
+      <c r="AQ11" s="335"/>
+      <c r="AR11" s="335"/>
+      <c r="AS11" s="335"/>
+      <c r="AT11" s="335"/>
+      <c r="AU11" s="335"/>
+      <c r="AV11" s="332"/>
+      <c r="AW11" s="335"/>
+      <c r="AX11" s="335"/>
       <c r="AY11" s="322" t="s">
         <v>88</v>
       </c>
@@ -8700,28 +8700,28 @@
       <c r="BA11" s="322" t="s">
         <v>90</v>
       </c>
-      <c r="BB11" s="333"/>
-      <c r="BC11" s="336"/>
-      <c r="BD11" s="336"/>
-      <c r="BE11" s="333"/>
-      <c r="BF11" s="333"/>
-      <c r="BG11" s="336"/>
-      <c r="BH11" s="336"/>
-      <c r="BI11" s="333"/>
-      <c r="BJ11" s="333"/>
-      <c r="BK11" s="333"/>
-      <c r="BL11" s="333"/>
-      <c r="BM11" s="336"/>
-      <c r="BN11" s="336"/>
-      <c r="BO11" s="336"/>
-      <c r="BP11" s="336"/>
-      <c r="BQ11" s="336"/>
-      <c r="BR11" s="336"/>
-      <c r="BS11" s="336"/>
-      <c r="BT11" s="333"/>
-      <c r="BU11" s="372"/>
+      <c r="BB11" s="332"/>
+      <c r="BC11" s="335"/>
+      <c r="BD11" s="335"/>
+      <c r="BE11" s="332"/>
+      <c r="BF11" s="332"/>
+      <c r="BG11" s="335"/>
+      <c r="BH11" s="335"/>
+      <c r="BI11" s="332"/>
+      <c r="BJ11" s="332"/>
+      <c r="BK11" s="332"/>
+      <c r="BL11" s="332"/>
+      <c r="BM11" s="335"/>
+      <c r="BN11" s="335"/>
+      <c r="BO11" s="335"/>
+      <c r="BP11" s="335"/>
+      <c r="BQ11" s="335"/>
+      <c r="BR11" s="335"/>
+      <c r="BS11" s="335"/>
+      <c r="BT11" s="332"/>
+      <c r="BU11" s="371"/>
       <c r="BV11" s="22"/>
-      <c r="BW11" s="349"/>
+      <c r="BW11" s="348"/>
       <c r="BX11" s="270" t="s">
         <v>91</v>
       </c>
@@ -8734,9 +8734,9 @@
       <c r="CA11" s="271" t="s">
         <v>94</v>
       </c>
-      <c r="CB11" s="379"/>
-      <c r="CC11" s="365"/>
-      <c r="CD11" s="365"/>
+      <c r="CB11" s="378"/>
+      <c r="CC11" s="364"/>
+      <c r="CD11" s="364"/>
       <c r="CE11" s="320">
         <v>26</v>
       </c>
@@ -9318,7 +9318,7 @@
       <c r="BK14" s="94"/>
       <c r="BL14" s="94">
         <f t="shared" ref="BL14:BQ14" si="6">SUM(BL15:BL21)</f>
-        <v>15756434</v>
+        <v>10172184</v>
       </c>
       <c r="BM14" s="94">
         <f t="shared" si="6"/>
@@ -9348,7 +9348,7 @@
       </c>
       <c r="BU14" s="316">
         <f>SUM(BU15:BU21)</f>
-        <v>129316973.6923077</v>
+        <v>134901223.69230768</v>
       </c>
       <c r="BV14" s="252"/>
       <c r="BW14" s="242"/>
@@ -9536,12 +9536,12 @@
         <v>95200</v>
       </c>
       <c r="BF15" s="280">
-        <f t="shared" ref="BF15:BF21" si="27">AM15+IF(E15="CT",IF(AR15&gt;=730000,730000,AR15),0)+IF(((AV15-AM15-IF(AR15&gt;=730000,730000,AR15)-AS15)*15%-AS15)&gt;"0",((AV15-AM15-IF(AR15&gt;=730000,730000,AR15)-AS15)*15%-AS15),0)</f>
-        <v>730000</v>
+        <f>AM15+IF(E15="CT",IF(AR15&gt;=730000,730000,AR15),0)+IF(((AV15-AM15-IF(AR15&gt;=730000,730000,AR15)-AS15)*15%-AS15)&gt;0,((AV15-AM15-IF(AR15&gt;=730000,730000,AR15)-AS15)*15%-AS15),0)</f>
+        <v>10220500</v>
       </c>
       <c r="BG15" s="280">
-        <f t="shared" ref="BG15:BG21" si="28">AV15-BF15+AW15</f>
-        <v>63270000</v>
+        <f t="shared" ref="BG15:BG21" si="27">AV15-BF15+AW15</f>
+        <v>53779500</v>
       </c>
       <c r="BH15" s="280">
         <v>3</v>
@@ -9554,12 +9554,12 @@
         <v>15500000</v>
       </c>
       <c r="BK15" s="280">
-        <f t="shared" ref="BK15:BK21" si="29">BG15-BB15-BC15+BD15-BH15*BI15-BJ15</f>
-        <v>28170400</v>
+        <f t="shared" ref="BK15:BK21" si="28">BG15-BB15-BC15+BD15-BH15*BI15-BJ15</f>
+        <v>18679900</v>
       </c>
       <c r="BL15" s="281">
-        <f t="shared" ref="BL15:BL21" si="30">IF(E15="TV",BK15*10%,IF(BK15&gt;0,ROUND(IF(BK15&gt;=80000000,BK15*35%-9850000,IF(BK15&gt;=52000000,BK15*30%-5850000,IF(BK15&gt;=32000000,BK15*25%-3250000,IF(BK15&gt;=18000000,BK15*20%-1650000,IF(BK15&gt;=10000000,BK15*15%-750000,IF(BK15&gt;5000000,BK15*10%-250000,BK15*5%)))))),0),0))</f>
-        <v>3984080</v>
+        <f t="shared" ref="BL15:BL21" si="29">IF(E15="TV",BK15*10%,IF(BK15&gt;0,ROUND(IF(BK15&gt;=80000000,BK15*35%-9850000,IF(BK15&gt;=52000000,BK15*30%-5850000,IF(BK15&gt;=32000000,BK15*25%-3250000,IF(BK15&gt;=18000000,BK15*20%-1650000,IF(BK15&gt;=10000000,BK15*15%-750000,IF(BK15&gt;5000000,BK15*10%-250000,BK15*5%)))))),0),0))</f>
+        <v>2085980</v>
       </c>
       <c r="BM15" s="280"/>
       <c r="BN15" s="280"/>
@@ -9570,12 +9570,12 @@
       <c r="BQ15" s="280"/>
       <c r="BR15" s="280"/>
       <c r="BS15" s="280"/>
-      <c r="BT15" s="330">
+      <c r="BT15" s="435">
         <v>25846153.846153852</v>
       </c>
       <c r="BU15" s="282">
-        <f t="shared" ref="BU15:BU21" si="31">AV15-BB15-BC15+BD15-BE15-BL15-BM15-BN15-BO15-BP15-BQ15-BR15+BS15-BT15</f>
-        <v>33074966.153846148</v>
+        <f t="shared" ref="BU15:BU21" si="30">AV15-BB15-BC15+BD15-BE15-BL15-BM15-BN15-BO15-BP15-BQ15-BR15+BS15-BT15</f>
+        <v>34973066.153846145</v>
       </c>
       <c r="BV15" s="252"/>
       <c r="BW15" s="283">
@@ -9589,11 +9589,11 @@
         <v>200000</v>
       </c>
       <c r="CA15" s="281">
-        <f t="shared" ref="CA15:CA21" si="32">+BW15*5%</f>
+        <f t="shared" ref="CA15:CA21" si="31">+BW15*5%</f>
         <v>3000000</v>
       </c>
       <c r="CB15" s="281">
-        <f t="shared" ref="CB15:CB21" si="33">SUM(BW15:CA15)</f>
+        <f t="shared" ref="CB15:CB21" si="32">SUM(BW15:CA15)</f>
         <v>63200000</v>
       </c>
       <c r="CC15" s="281"/>
@@ -9733,7 +9733,7 @@
         <v>0</v>
       </c>
       <c r="AN16" s="94">
-        <f t="shared" ref="AN16:AN21" si="34">H16/26*K16</f>
+        <f t="shared" ref="AN16:AN21" si="33">H16/26*K16</f>
         <v>0</v>
       </c>
       <c r="AO16" s="94">
@@ -9779,29 +9779,29 @@
         <f t="shared" si="26"/>
         <v>84800</v>
       </c>
-      <c r="BF16" s="250">
+      <c r="BF16" s="434">
+        <f t="shared" ref="BF16:BF21" si="34">AM16+IF(E16="CT",IF(AR16&gt;=730000,730000,AR16),0)+IF(((AV16-AM16-IF(AR16&gt;=730000,730000,AR16)-AS16)*15%-AS16)&gt;0,((AV16-AM16-IF(AR16&gt;=730000,730000,AR16)-AS16)*15%-AS16),0)</f>
+        <v>7925769.230769231</v>
+      </c>
+      <c r="BG16" s="250">
         <f t="shared" si="27"/>
-        <v>720000</v>
-      </c>
-      <c r="BG16" s="250">
-        <f t="shared" si="28"/>
-        <v>48038461.538461544</v>
+        <v>40832692.307692312</v>
       </c>
       <c r="BH16" s="250"/>
       <c r="BI16" s="280">
         <v>6200000</v>
       </c>
-      <c r="BJ16" s="435">
+      <c r="BJ16" s="434">
         <f t="shared" ref="BJ16:BJ21" si="35">IF(E16="CT",15500000,0)</f>
         <v>15500000</v>
       </c>
       <c r="BK16" s="250">
+        <f t="shared" si="28"/>
+        <v>24442292.307692312</v>
+      </c>
+      <c r="BL16" s="243">
         <f t="shared" si="29"/>
-        <v>31648061.538461544</v>
-      </c>
-      <c r="BL16" s="243">
-        <f t="shared" si="30"/>
-        <v>4679612</v>
+        <v>3238458</v>
       </c>
       <c r="BM16" s="250"/>
       <c r="BN16" s="250"/>
@@ -9816,8 +9816,8 @@
         <v>0</v>
       </c>
       <c r="BU16" s="251">
-        <f t="shared" si="31"/>
-        <v>43103649.538461544</v>
+        <f t="shared" si="30"/>
+        <v>44544803.538461544</v>
       </c>
       <c r="BV16" s="252"/>
       <c r="BW16" s="242">
@@ -9833,11 +9833,11 @@
         <v>200000</v>
       </c>
       <c r="CA16" s="243">
+        <f t="shared" si="31"/>
+        <v>2000000</v>
+      </c>
+      <c r="CB16" s="243">
         <f t="shared" si="32"/>
-        <v>2000000</v>
-      </c>
-      <c r="CB16" s="243">
-        <f t="shared" si="33"/>
         <v>52200000</v>
       </c>
       <c r="CC16" s="243"/>
@@ -9977,7 +9977,7 @@
         <v>0</v>
       </c>
       <c r="AN17" s="94">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>0</v>
       </c>
       <c r="AO17" s="94">
@@ -10023,29 +10023,29 @@
         <f t="shared" si="26"/>
         <v>78200</v>
       </c>
-      <c r="BF17" s="250">
+      <c r="BF17" s="434">
+        <f t="shared" si="34"/>
+        <v>6862307.692307692</v>
+      </c>
+      <c r="BG17" s="250">
         <f t="shared" si="27"/>
-        <v>560000</v>
-      </c>
-      <c r="BG17" s="250">
-        <f t="shared" si="28"/>
-        <v>42015384.615384616</v>
+        <v>35713076.923076928</v>
       </c>
       <c r="BH17" s="250"/>
       <c r="BI17" s="280">
         <v>6200000</v>
       </c>
-      <c r="BJ17" s="435">
+      <c r="BJ17" s="434">
         <f t="shared" si="35"/>
         <v>15500000</v>
       </c>
       <c r="BK17" s="250">
+        <f t="shared" si="28"/>
+        <v>19391976.923076928</v>
+      </c>
+      <c r="BL17" s="243">
         <f t="shared" si="29"/>
-        <v>25694284.615384616</v>
-      </c>
-      <c r="BL17" s="243">
-        <f t="shared" si="30"/>
-        <v>3488857</v>
+        <v>2228395</v>
       </c>
       <c r="BM17" s="250"/>
       <c r="BN17" s="250"/>
@@ -10060,8 +10060,8 @@
         <v>25846153.846153852</v>
       </c>
       <c r="BU17" s="251">
-        <f t="shared" si="31"/>
-        <v>12341073.769230764</v>
+        <f t="shared" si="30"/>
+        <v>13601535.769230764</v>
       </c>
       <c r="BV17" s="252"/>
       <c r="BW17" s="242">
@@ -10077,11 +10077,11 @@
         <v>200000</v>
       </c>
       <c r="CA17" s="243">
+        <f t="shared" si="31"/>
+        <v>2000000</v>
+      </c>
+      <c r="CB17" s="243">
         <f t="shared" si="32"/>
-        <v>2000000</v>
-      </c>
-      <c r="CB17" s="243">
-        <f t="shared" si="33"/>
         <v>42200000</v>
       </c>
       <c r="CC17" s="243"/>
@@ -10221,7 +10221,7 @@
         <v>0</v>
       </c>
       <c r="AN18" s="94">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>0</v>
       </c>
       <c r="AO18" s="94">
@@ -10267,29 +10267,29 @@
         <f t="shared" si="26"/>
         <v>69900</v>
       </c>
-      <c r="BF18" s="250">
+      <c r="BF18" s="434">
+        <f t="shared" si="34"/>
+        <v>4645961.538461538</v>
+      </c>
+      <c r="BG18" s="250">
         <f t="shared" si="27"/>
-        <v>720000</v>
-      </c>
-      <c r="BG18" s="250">
-        <f t="shared" si="28"/>
-        <v>26173076.923076924</v>
+        <v>22247115.384615384</v>
       </c>
       <c r="BH18" s="250"/>
       <c r="BI18" s="280">
         <v>6200000</v>
       </c>
-      <c r="BJ18" s="435">
+      <c r="BJ18" s="434">
         <f t="shared" si="35"/>
         <v>15500000</v>
       </c>
       <c r="BK18" s="250">
+        <f t="shared" si="28"/>
+        <v>6013165.384615384</v>
+      </c>
+      <c r="BL18" s="243">
         <f t="shared" si="29"/>
-        <v>9939126.9230769239</v>
-      </c>
-      <c r="BL18" s="243">
-        <f t="shared" si="30"/>
-        <v>743913</v>
+        <v>351317</v>
       </c>
       <c r="BM18" s="250"/>
       <c r="BN18" s="250"/>
@@ -10304,8 +10304,8 @@
         <v>10195307.692307694</v>
       </c>
       <c r="BU18" s="251">
-        <f t="shared" si="31"/>
-        <v>15150006.23076923</v>
+        <f t="shared" si="30"/>
+        <v>15542602.23076923</v>
       </c>
       <c r="BV18" s="252"/>
       <c r="BW18" s="242">
@@ -10321,11 +10321,11 @@
         <v>200000</v>
       </c>
       <c r="CA18" s="243">
+        <f t="shared" si="31"/>
+        <v>1150000</v>
+      </c>
+      <c r="CB18" s="243">
         <f t="shared" si="32"/>
-        <v>1150000</v>
-      </c>
-      <c r="CB18" s="243">
-        <f t="shared" si="33"/>
         <v>26350000</v>
       </c>
       <c r="CC18" s="243"/>
@@ -10465,7 +10465,7 @@
         <v>0</v>
       </c>
       <c r="AN19" s="94">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>0</v>
       </c>
       <c r="AO19" s="94">
@@ -10511,28 +10511,28 @@
         <f t="shared" si="26"/>
         <v>48500</v>
       </c>
-      <c r="BF19" s="250">
+      <c r="BF19" s="434">
+        <f t="shared" si="34"/>
+        <v>2303461.5384615385</v>
+      </c>
+      <c r="BG19" s="250">
         <f t="shared" si="27"/>
-        <v>560000</v>
-      </c>
-      <c r="BG19" s="250">
-        <f t="shared" si="28"/>
-        <v>11623076.923076924</v>
+        <v>9879615.3846153859</v>
       </c>
       <c r="BH19" s="250"/>
       <c r="BI19" s="280">
         <v>6200000</v>
       </c>
-      <c r="BJ19" s="435">
+      <c r="BJ19" s="434">
         <f t="shared" si="35"/>
         <v>15500000</v>
       </c>
       <c r="BK19" s="250">
+        <f t="shared" si="28"/>
+        <v>-6129634.6153846141</v>
+      </c>
+      <c r="BL19" s="243">
         <f t="shared" si="29"/>
-        <v>-4386173.0769230761</v>
-      </c>
-      <c r="BL19" s="243">
-        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="BM19" s="250"/>
@@ -10548,7 +10548,7 @@
         <v>9977846.153846154</v>
       </c>
       <c r="BU19" s="251">
-        <f t="shared" si="31"/>
+        <f t="shared" si="30"/>
         <v>1647480.7692307699</v>
       </c>
       <c r="BV19" s="252"/>
@@ -10565,11 +10565,11 @@
         <v>200000</v>
       </c>
       <c r="CA19" s="243">
+        <f t="shared" si="31"/>
+        <v>550000</v>
+      </c>
+      <c r="CB19" s="243">
         <f t="shared" si="32"/>
-        <v>550000</v>
-      </c>
-      <c r="CB19" s="243">
-        <f t="shared" si="33"/>
         <v>11750000</v>
       </c>
       <c r="CC19" s="243"/>
@@ -10709,7 +10709,7 @@
         <v>0</v>
       </c>
       <c r="AN20" s="94">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>0</v>
       </c>
       <c r="AO20" s="94">
@@ -10755,29 +10755,29 @@
         <f t="shared" si="26"/>
         <v>63400</v>
       </c>
-      <c r="BF20" s="250">
+      <c r="BF20" s="434">
+        <f t="shared" si="34"/>
+        <v>3622500</v>
+      </c>
+      <c r="BG20" s="250">
         <f t="shared" si="27"/>
-        <v>0</v>
-      </c>
-      <c r="BG20" s="250">
-        <f t="shared" si="28"/>
-        <v>24870000</v>
+        <v>21247500</v>
       </c>
       <c r="BH20" s="250"/>
       <c r="BI20" s="280">
         <v>6200000</v>
       </c>
-      <c r="BJ20" s="435">
+      <c r="BJ20" s="434">
         <f t="shared" si="35"/>
         <v>0</v>
       </c>
       <c r="BK20" s="250">
+        <f t="shared" si="28"/>
+        <v>21247500</v>
+      </c>
+      <c r="BL20" s="243">
         <f t="shared" si="29"/>
-        <v>24870000</v>
-      </c>
-      <c r="BL20" s="243">
-        <f t="shared" si="30"/>
-        <v>2487000</v>
+        <v>2124750</v>
       </c>
       <c r="BM20" s="250"/>
       <c r="BN20" s="250"/>
@@ -10792,8 +10792,8 @@
         <v>10195307.692307694</v>
       </c>
       <c r="BU20" s="251">
-        <f t="shared" si="31"/>
-        <v>12124292.307692306</v>
+        <f t="shared" si="30"/>
+        <v>12486542.307692306</v>
       </c>
       <c r="BV20" s="252"/>
       <c r="BW20" s="242">
@@ -10809,11 +10809,11 @@
         <v>200000</v>
       </c>
       <c r="CA20" s="243">
+        <f t="shared" si="31"/>
+        <v>1150000</v>
+      </c>
+      <c r="CB20" s="243">
         <f t="shared" si="32"/>
-        <v>1150000</v>
-      </c>
-      <c r="CB20" s="243">
-        <f t="shared" si="33"/>
         <v>24350000</v>
       </c>
       <c r="CC20" s="243" t="s">
@@ -10955,7 +10955,7 @@
         <v>0</v>
       </c>
       <c r="AN21" s="94">
-        <f t="shared" si="34"/>
+        <f t="shared" si="33"/>
         <v>300000</v>
       </c>
       <c r="AO21" s="94">
@@ -11001,29 +11001,29 @@
         <f t="shared" si="26"/>
         <v>63400</v>
       </c>
-      <c r="BF21" s="250">
+      <c r="BF21" s="434">
+        <f t="shared" si="34"/>
+        <v>3924038.4615384615</v>
+      </c>
+      <c r="BG21" s="250">
         <f t="shared" si="27"/>
-        <v>560000</v>
-      </c>
-      <c r="BG21" s="250">
-        <f t="shared" si="28"/>
-        <v>22426923.076923076</v>
+        <v>19062884.615384616</v>
       </c>
       <c r="BH21" s="250"/>
       <c r="BI21" s="280">
         <v>6200000</v>
       </c>
-      <c r="BJ21" s="435">
+      <c r="BJ21" s="434">
         <f t="shared" si="35"/>
         <v>15500000</v>
       </c>
       <c r="BK21" s="250">
+        <f t="shared" si="28"/>
+        <v>2865684.615384616</v>
+      </c>
+      <c r="BL21" s="243">
         <f t="shared" si="29"/>
-        <v>6229723.0769230761</v>
-      </c>
-      <c r="BL21" s="243">
-        <f t="shared" si="30"/>
-        <v>372972</v>
+        <v>143284</v>
       </c>
       <c r="BM21" s="250"/>
       <c r="BN21" s="250"/>
@@ -11038,8 +11038,8 @@
         <v>9977846.153846154</v>
       </c>
       <c r="BU21" s="251">
-        <f t="shared" si="31"/>
-        <v>11875504.923076922</v>
+        <f t="shared" si="30"/>
+        <v>12105192.923076922</v>
       </c>
       <c r="BV21" s="252"/>
       <c r="BW21" s="242">
@@ -11055,11 +11055,11 @@
         <v>200000</v>
       </c>
       <c r="CA21" s="243">
+        <f t="shared" si="31"/>
+        <v>850000</v>
+      </c>
+      <c r="CB21" s="243">
         <f t="shared" si="32"/>
-        <v>850000</v>
-      </c>
-      <c r="CB21" s="243">
-        <f t="shared" si="33"/>
         <v>18050000</v>
       </c>
       <c r="CC21" s="243" t="s">
@@ -11500,87 +11500,87 @@
       <c r="CD2" s="132"/>
     </row>
     <row r="3" spans="1:87" s="134" customFormat="1" ht="11" outlineLevel="1">
-      <c r="A3" s="416"/>
-      <c r="B3" s="404"/>
-      <c r="C3" s="404"/>
-      <c r="D3" s="404"/>
-      <c r="E3" s="404"/>
-      <c r="F3" s="404"/>
-      <c r="G3" s="404"/>
-      <c r="H3" s="404"/>
-      <c r="I3" s="404"/>
-      <c r="J3" s="404"/>
-      <c r="K3" s="404"/>
-      <c r="L3" s="404"/>
-      <c r="M3" s="404"/>
-      <c r="N3" s="404"/>
-      <c r="O3" s="404"/>
-      <c r="P3" s="404"/>
-      <c r="Q3" s="404"/>
-      <c r="R3" s="404"/>
-      <c r="S3" s="404"/>
-      <c r="T3" s="404"/>
-      <c r="U3" s="404"/>
-      <c r="V3" s="404"/>
-      <c r="W3" s="404"/>
-      <c r="X3" s="404"/>
-      <c r="Y3" s="404"/>
-      <c r="Z3" s="404"/>
-      <c r="AA3" s="404"/>
-      <c r="AB3" s="404"/>
-      <c r="AC3" s="404"/>
-      <c r="AD3" s="404"/>
-      <c r="AE3" s="404"/>
-      <c r="AF3" s="404"/>
-      <c r="AG3" s="404"/>
-      <c r="AH3" s="404"/>
-      <c r="AI3" s="404"/>
-      <c r="AJ3" s="404"/>
-      <c r="AK3" s="404"/>
-      <c r="AL3" s="404"/>
-      <c r="AM3" s="404"/>
-      <c r="AN3" s="404"/>
-      <c r="AO3" s="404"/>
-      <c r="AP3" s="404"/>
-      <c r="AQ3" s="404"/>
-      <c r="AR3" s="404"/>
-      <c r="AS3" s="404"/>
-      <c r="AT3" s="404"/>
-      <c r="AU3" s="404"/>
-      <c r="AV3" s="404"/>
-      <c r="AW3" s="404"/>
-      <c r="AX3" s="404"/>
-      <c r="AY3" s="404"/>
-      <c r="AZ3" s="404"/>
-      <c r="BA3" s="404"/>
-      <c r="BB3" s="404"/>
-      <c r="BC3" s="404"/>
-      <c r="BD3" s="404"/>
-      <c r="BE3" s="404"/>
-      <c r="BF3" s="404"/>
-      <c r="BG3" s="404"/>
-      <c r="BH3" s="404"/>
-      <c r="BI3" s="404"/>
-      <c r="BJ3" s="404"/>
-      <c r="BK3" s="404"/>
-      <c r="BL3" s="404"/>
-      <c r="BM3" s="404"/>
-      <c r="BN3" s="404"/>
-      <c r="BO3" s="404"/>
-      <c r="BP3" s="404"/>
-      <c r="BQ3" s="404"/>
-      <c r="BR3" s="404"/>
-      <c r="BS3" s="404"/>
-      <c r="BT3" s="404"/>
-      <c r="BU3" s="404"/>
-      <c r="BW3" s="403" t="s">
+      <c r="A3" s="415"/>
+      <c r="B3" s="403"/>
+      <c r="C3" s="403"/>
+      <c r="D3" s="403"/>
+      <c r="E3" s="403"/>
+      <c r="F3" s="403"/>
+      <c r="G3" s="403"/>
+      <c r="H3" s="403"/>
+      <c r="I3" s="403"/>
+      <c r="J3" s="403"/>
+      <c r="K3" s="403"/>
+      <c r="L3" s="403"/>
+      <c r="M3" s="403"/>
+      <c r="N3" s="403"/>
+      <c r="O3" s="403"/>
+      <c r="P3" s="403"/>
+      <c r="Q3" s="403"/>
+      <c r="R3" s="403"/>
+      <c r="S3" s="403"/>
+      <c r="T3" s="403"/>
+      <c r="U3" s="403"/>
+      <c r="V3" s="403"/>
+      <c r="W3" s="403"/>
+      <c r="X3" s="403"/>
+      <c r="Y3" s="403"/>
+      <c r="Z3" s="403"/>
+      <c r="AA3" s="403"/>
+      <c r="AB3" s="403"/>
+      <c r="AC3" s="403"/>
+      <c r="AD3" s="403"/>
+      <c r="AE3" s="403"/>
+      <c r="AF3" s="403"/>
+      <c r="AG3" s="403"/>
+      <c r="AH3" s="403"/>
+      <c r="AI3" s="403"/>
+      <c r="AJ3" s="403"/>
+      <c r="AK3" s="403"/>
+      <c r="AL3" s="403"/>
+      <c r="AM3" s="403"/>
+      <c r="AN3" s="403"/>
+      <c r="AO3" s="403"/>
+      <c r="AP3" s="403"/>
+      <c r="AQ3" s="403"/>
+      <c r="AR3" s="403"/>
+      <c r="AS3" s="403"/>
+      <c r="AT3" s="403"/>
+      <c r="AU3" s="403"/>
+      <c r="AV3" s="403"/>
+      <c r="AW3" s="403"/>
+      <c r="AX3" s="403"/>
+      <c r="AY3" s="403"/>
+      <c r="AZ3" s="403"/>
+      <c r="BA3" s="403"/>
+      <c r="BB3" s="403"/>
+      <c r="BC3" s="403"/>
+      <c r="BD3" s="403"/>
+      <c r="BE3" s="403"/>
+      <c r="BF3" s="403"/>
+      <c r="BG3" s="403"/>
+      <c r="BH3" s="403"/>
+      <c r="BI3" s="403"/>
+      <c r="BJ3" s="403"/>
+      <c r="BK3" s="403"/>
+      <c r="BL3" s="403"/>
+      <c r="BM3" s="403"/>
+      <c r="BN3" s="403"/>
+      <c r="BO3" s="403"/>
+      <c r="BP3" s="403"/>
+      <c r="BQ3" s="403"/>
+      <c r="BR3" s="403"/>
+      <c r="BS3" s="403"/>
+      <c r="BT3" s="403"/>
+      <c r="BU3" s="403"/>
+      <c r="BW3" s="402" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="404"/>
-      <c r="BY3" s="404"/>
-      <c r="BZ3" s="404"/>
-      <c r="CA3" s="404"/>
-      <c r="CB3" s="404"/>
+      <c r="BX3" s="403"/>
+      <c r="BY3" s="403"/>
+      <c r="BZ3" s="403"/>
+      <c r="CA3" s="403"/>
+      <c r="CB3" s="403"/>
       <c r="CC3" s="133"/>
       <c r="CD3" s="133"/>
       <c r="CE3" s="134" t="s">
@@ -11663,364 +11663,364 @@
       <c r="BS4" s="135"/>
       <c r="BT4" s="135"/>
       <c r="BU4" s="135"/>
-      <c r="BW4" s="404"/>
-      <c r="BX4" s="404"/>
-      <c r="BY4" s="404"/>
-      <c r="BZ4" s="404"/>
-      <c r="CA4" s="404"/>
-      <c r="CB4" s="404"/>
+      <c r="BW4" s="403"/>
+      <c r="BX4" s="403"/>
+      <c r="BY4" s="403"/>
+      <c r="BZ4" s="403"/>
+      <c r="CA4" s="403"/>
+      <c r="CB4" s="403"/>
       <c r="CC4" s="133"/>
       <c r="CD4" s="133"/>
     </row>
     <row r="5" spans="1:87" s="136" customFormat="1">
-      <c r="A5" s="392" t="s">
+      <c r="A5" s="391" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="402" t="s">
+      <c r="B5" s="401" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="390" t="s">
+      <c r="C5" s="389" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="398" t="s">
+      <c r="D5" s="397" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="398" t="s">
+      <c r="E5" s="397" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="390" t="s">
+      <c r="F5" s="389" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="390" t="s">
+      <c r="G5" s="389" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="346" t="s">
+      <c r="H5" s="345" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="346" t="s">
+      <c r="I5" s="345" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="390" t="s">
+      <c r="J5" s="389" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="396" t="s">
+      <c r="K5" s="395" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="387"/>
-      <c r="M5" s="387"/>
-      <c r="N5" s="387"/>
-      <c r="O5" s="387"/>
-      <c r="P5" s="387"/>
-      <c r="Q5" s="387"/>
-      <c r="R5" s="387"/>
-      <c r="S5" s="387"/>
-      <c r="T5" s="387"/>
-      <c r="U5" s="387"/>
-      <c r="V5" s="387"/>
-      <c r="W5" s="387"/>
-      <c r="X5" s="387"/>
-      <c r="Y5" s="390" t="s">
+      <c r="L5" s="386"/>
+      <c r="M5" s="386"/>
+      <c r="N5" s="386"/>
+      <c r="O5" s="386"/>
+      <c r="P5" s="386"/>
+      <c r="Q5" s="386"/>
+      <c r="R5" s="386"/>
+      <c r="S5" s="386"/>
+      <c r="T5" s="386"/>
+      <c r="U5" s="386"/>
+      <c r="V5" s="386"/>
+      <c r="W5" s="386"/>
+      <c r="X5" s="386"/>
+      <c r="Y5" s="389" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="387"/>
-      <c r="AA5" s="387"/>
-      <c r="AB5" s="387"/>
-      <c r="AC5" s="387"/>
-      <c r="AD5" s="387"/>
-      <c r="AE5" s="387"/>
-      <c r="AF5" s="387"/>
-      <c r="AG5" s="387"/>
-      <c r="AH5" s="387"/>
-      <c r="AI5" s="387"/>
-      <c r="AJ5" s="387"/>
-      <c r="AK5" s="387"/>
-      <c r="AL5" s="387"/>
-      <c r="AM5" s="387"/>
-      <c r="AN5" s="387"/>
-      <c r="AO5" s="388"/>
-      <c r="AP5" s="390" t="s">
+      <c r="Z5" s="386"/>
+      <c r="AA5" s="386"/>
+      <c r="AB5" s="386"/>
+      <c r="AC5" s="386"/>
+      <c r="AD5" s="386"/>
+      <c r="AE5" s="386"/>
+      <c r="AF5" s="386"/>
+      <c r="AG5" s="386"/>
+      <c r="AH5" s="386"/>
+      <c r="AI5" s="386"/>
+      <c r="AJ5" s="386"/>
+      <c r="AK5" s="386"/>
+      <c r="AL5" s="386"/>
+      <c r="AM5" s="386"/>
+      <c r="AN5" s="386"/>
+      <c r="AO5" s="387"/>
+      <c r="AP5" s="389" t="s">
         <v>16</v>
       </c>
-      <c r="AQ5" s="390" t="s">
+      <c r="AQ5" s="389" t="s">
         <v>17</v>
       </c>
-      <c r="AR5" s="390" t="s">
+      <c r="AR5" s="389" t="s">
         <v>18</v>
       </c>
-      <c r="AS5" s="390" t="s">
+      <c r="AS5" s="389" t="s">
         <v>19</v>
       </c>
-      <c r="AT5" s="390" t="s">
+      <c r="AT5" s="389" t="s">
         <v>20</v>
       </c>
-      <c r="AU5" s="390" t="s">
+      <c r="AU5" s="389" t="s">
         <v>21</v>
       </c>
-      <c r="AV5" s="390" t="s">
+      <c r="AV5" s="389" t="s">
         <v>22</v>
       </c>
-      <c r="AW5" s="390" t="s">
+      <c r="AW5" s="389" t="s">
         <v>23</v>
       </c>
-      <c r="AX5" s="390" t="s">
+      <c r="AX5" s="389" t="s">
         <v>24</v>
       </c>
-      <c r="AY5" s="386" t="s">
+      <c r="AY5" s="385" t="s">
         <v>25</v>
       </c>
-      <c r="AZ5" s="387"/>
-      <c r="BA5" s="387"/>
-      <c r="BB5" s="387"/>
-      <c r="BC5" s="387"/>
-      <c r="BD5" s="387"/>
-      <c r="BE5" s="387"/>
-      <c r="BF5" s="387"/>
-      <c r="BG5" s="387"/>
-      <c r="BH5" s="387"/>
-      <c r="BI5" s="387"/>
-      <c r="BJ5" s="387"/>
-      <c r="BK5" s="387"/>
-      <c r="BL5" s="387"/>
-      <c r="BM5" s="387"/>
-      <c r="BN5" s="387"/>
-      <c r="BO5" s="387"/>
-      <c r="BP5" s="387"/>
-      <c r="BQ5" s="388"/>
-      <c r="BR5" s="407" t="s">
+      <c r="AZ5" s="386"/>
+      <c r="BA5" s="386"/>
+      <c r="BB5" s="386"/>
+      <c r="BC5" s="386"/>
+      <c r="BD5" s="386"/>
+      <c r="BE5" s="386"/>
+      <c r="BF5" s="386"/>
+      <c r="BG5" s="386"/>
+      <c r="BH5" s="386"/>
+      <c r="BI5" s="386"/>
+      <c r="BJ5" s="386"/>
+      <c r="BK5" s="386"/>
+      <c r="BL5" s="386"/>
+      <c r="BM5" s="386"/>
+      <c r="BN5" s="386"/>
+      <c r="BO5" s="386"/>
+      <c r="BP5" s="386"/>
+      <c r="BQ5" s="387"/>
+      <c r="BR5" s="406" t="s">
         <v>26</v>
       </c>
-      <c r="BS5" s="400"/>
-      <c r="BT5" s="386" t="s">
+      <c r="BS5" s="399"/>
+      <c r="BT5" s="385" t="s">
         <v>27</v>
       </c>
-      <c r="BU5" s="418" t="s">
+      <c r="BU5" s="417" t="s">
         <v>28</v>
       </c>
-      <c r="BW5" s="419" t="s">
+      <c r="BW5" s="418" t="s">
         <v>29</v>
       </c>
-      <c r="BX5" s="408" t="s">
+      <c r="BX5" s="407" t="s">
         <v>30</v>
       </c>
-      <c r="BY5" s="409"/>
-      <c r="BZ5" s="409"/>
-      <c r="CA5" s="400"/>
-      <c r="CB5" s="420" t="s">
+      <c r="BY5" s="408"/>
+      <c r="BZ5" s="408"/>
+      <c r="CA5" s="399"/>
+      <c r="CB5" s="419" t="s">
         <v>31</v>
       </c>
-      <c r="CC5" s="405" t="s">
+      <c r="CC5" s="404" t="s">
         <v>32</v>
       </c>
-      <c r="CD5" s="405" t="s">
+      <c r="CD5" s="404" t="s">
         <v>33</v>
       </c>
       <c r="CH5" s="137"/>
       <c r="CI5" s="138"/>
     </row>
     <row r="6" spans="1:87" s="136" customFormat="1">
-      <c r="A6" s="384"/>
-      <c r="B6" s="384"/>
-      <c r="C6" s="384"/>
-      <c r="D6" s="384"/>
-      <c r="E6" s="384"/>
-      <c r="F6" s="384"/>
-      <c r="G6" s="384"/>
-      <c r="H6" s="384"/>
-      <c r="I6" s="384"/>
-      <c r="J6" s="384"/>
-      <c r="K6" s="391" t="s">
+      <c r="A6" s="383"/>
+      <c r="B6" s="383"/>
+      <c r="C6" s="383"/>
+      <c r="D6" s="383"/>
+      <c r="E6" s="383"/>
+      <c r="F6" s="383"/>
+      <c r="G6" s="383"/>
+      <c r="H6" s="383"/>
+      <c r="I6" s="383"/>
+      <c r="J6" s="383"/>
+      <c r="K6" s="390" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="391" t="s">
+      <c r="L6" s="390" t="s">
         <v>35</v>
       </c>
-      <c r="M6" s="391" t="s">
+      <c r="M6" s="390" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="391" t="s">
+      <c r="N6" s="390" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="391" t="s">
+      <c r="O6" s="390" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="391" t="s">
+      <c r="P6" s="390" t="s">
         <v>39</v>
       </c>
-      <c r="Q6" s="391" t="s">
+      <c r="Q6" s="390" t="s">
         <v>40</v>
       </c>
-      <c r="R6" s="391" t="s">
+      <c r="R6" s="390" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="391" t="s">
+      <c r="S6" s="390" t="s">
         <v>42</v>
       </c>
-      <c r="T6" s="391" t="s">
+      <c r="T6" s="390" t="s">
         <v>43</v>
       </c>
-      <c r="U6" s="391" t="s">
+      <c r="U6" s="390" t="s">
         <v>44</v>
       </c>
-      <c r="V6" s="399" t="s">
+      <c r="V6" s="398" t="s">
         <v>45</v>
       </c>
-      <c r="W6" s="400"/>
-      <c r="X6" s="391" t="s">
+      <c r="W6" s="399"/>
+      <c r="X6" s="390" t="s">
         <v>46</v>
       </c>
-      <c r="Y6" s="390" t="s">
+      <c r="Y6" s="389" t="s">
         <v>47</v>
       </c>
-      <c r="Z6" s="390" t="s">
+      <c r="Z6" s="389" t="s">
         <v>48</v>
       </c>
-      <c r="AA6" s="390" t="s">
+      <c r="AA6" s="389" t="s">
         <v>49</v>
       </c>
-      <c r="AB6" s="390" t="s">
+      <c r="AB6" s="389" t="s">
         <v>50</v>
       </c>
-      <c r="AC6" s="346" t="s">
+      <c r="AC6" s="345" t="s">
         <v>51</v>
       </c>
-      <c r="AD6" s="346" t="s">
+      <c r="AD6" s="345" t="s">
         <v>52</v>
       </c>
-      <c r="AE6" s="346" t="s">
+      <c r="AE6" s="345" t="s">
         <v>53</v>
       </c>
-      <c r="AF6" s="346" t="s">
+      <c r="AF6" s="345" t="s">
         <v>54</v>
       </c>
-      <c r="AG6" s="390" t="s">
+      <c r="AG6" s="389" t="s">
         <v>55</v>
       </c>
-      <c r="AH6" s="346" t="s">
+      <c r="AH6" s="345" t="s">
         <v>56</v>
       </c>
-      <c r="AI6" s="346" t="s">
+      <c r="AI6" s="345" t="s">
         <v>57</v>
       </c>
-      <c r="AJ6" s="390" t="s">
+      <c r="AJ6" s="389" t="s">
         <v>58</v>
       </c>
-      <c r="AK6" s="393" t="s">
+      <c r="AK6" s="392" t="s">
         <v>59</v>
       </c>
-      <c r="AL6" s="390" t="s">
+      <c r="AL6" s="389" t="s">
         <v>60</v>
       </c>
-      <c r="AM6" s="390" t="s">
+      <c r="AM6" s="389" t="s">
         <v>61</v>
       </c>
-      <c r="AN6" s="397" t="s">
+      <c r="AN6" s="396" t="s">
         <v>62</v>
       </c>
-      <c r="AO6" s="390" t="s">
+      <c r="AO6" s="389" t="s">
         <v>63</v>
       </c>
-      <c r="AP6" s="384"/>
-      <c r="AQ6" s="384"/>
-      <c r="AR6" s="384"/>
-      <c r="AS6" s="384"/>
-      <c r="AT6" s="384"/>
-      <c r="AU6" s="384"/>
-      <c r="AV6" s="384"/>
-      <c r="AW6" s="384"/>
-      <c r="AX6" s="384"/>
-      <c r="AY6" s="386" t="s">
+      <c r="AP6" s="383"/>
+      <c r="AQ6" s="383"/>
+      <c r="AR6" s="383"/>
+      <c r="AS6" s="383"/>
+      <c r="AT6" s="383"/>
+      <c r="AU6" s="383"/>
+      <c r="AV6" s="383"/>
+      <c r="AW6" s="383"/>
+      <c r="AX6" s="383"/>
+      <c r="AY6" s="385" t="s">
         <v>25</v>
       </c>
-      <c r="AZ6" s="387"/>
-      <c r="BA6" s="387"/>
-      <c r="BB6" s="387"/>
-      <c r="BC6" s="387"/>
-      <c r="BD6" s="387"/>
-      <c r="BE6" s="387"/>
-      <c r="BF6" s="387"/>
-      <c r="BG6" s="387"/>
-      <c r="BH6" s="387"/>
-      <c r="BI6" s="387"/>
-      <c r="BJ6" s="387"/>
-      <c r="BK6" s="387"/>
-      <c r="BL6" s="388"/>
-      <c r="BM6" s="386" t="s">
+      <c r="AZ6" s="386"/>
+      <c r="BA6" s="386"/>
+      <c r="BB6" s="386"/>
+      <c r="BC6" s="386"/>
+      <c r="BD6" s="386"/>
+      <c r="BE6" s="386"/>
+      <c r="BF6" s="386"/>
+      <c r="BG6" s="386"/>
+      <c r="BH6" s="386"/>
+      <c r="BI6" s="386"/>
+      <c r="BJ6" s="386"/>
+      <c r="BK6" s="386"/>
+      <c r="BL6" s="387"/>
+      <c r="BM6" s="385" t="s">
         <v>64</v>
       </c>
-      <c r="BN6" s="387"/>
-      <c r="BO6" s="387"/>
-      <c r="BP6" s="387"/>
-      <c r="BQ6" s="388"/>
-      <c r="BR6" s="383" t="s">
+      <c r="BN6" s="386"/>
+      <c r="BO6" s="386"/>
+      <c r="BP6" s="386"/>
+      <c r="BQ6" s="387"/>
+      <c r="BR6" s="382" t="s">
         <v>65</v>
       </c>
-      <c r="BS6" s="383" t="s">
+      <c r="BS6" s="382" t="s">
         <v>66</v>
       </c>
-      <c r="BT6" s="384"/>
-      <c r="BU6" s="394"/>
-      <c r="BW6" s="411"/>
-      <c r="BX6" s="394"/>
-      <c r="BY6" s="410"/>
-      <c r="BZ6" s="410"/>
-      <c r="CA6" s="411"/>
-      <c r="CB6" s="384"/>
-      <c r="CC6" s="384"/>
-      <c r="CD6" s="384"/>
+      <c r="BT6" s="383"/>
+      <c r="BU6" s="393"/>
+      <c r="BW6" s="410"/>
+      <c r="BX6" s="393"/>
+      <c r="BY6" s="409"/>
+      <c r="BZ6" s="409"/>
+      <c r="CA6" s="410"/>
+      <c r="CB6" s="383"/>
+      <c r="CC6" s="383"/>
+      <c r="CD6" s="383"/>
       <c r="CH6" s="137"/>
       <c r="CI6" s="138"/>
     </row>
     <row r="7" spans="1:87" s="139" customFormat="1" ht="12">
-      <c r="A7" s="384"/>
-      <c r="B7" s="384"/>
-      <c r="C7" s="384"/>
-      <c r="D7" s="384"/>
-      <c r="E7" s="384"/>
-      <c r="F7" s="384"/>
-      <c r="G7" s="384"/>
-      <c r="H7" s="384"/>
-      <c r="I7" s="384"/>
-      <c r="J7" s="384"/>
-      <c r="K7" s="384"/>
-      <c r="L7" s="384"/>
-      <c r="M7" s="384"/>
-      <c r="N7" s="384"/>
-      <c r="O7" s="384"/>
-      <c r="P7" s="384"/>
-      <c r="Q7" s="384"/>
-      <c r="R7" s="384"/>
-      <c r="S7" s="384"/>
-      <c r="T7" s="384"/>
-      <c r="U7" s="384"/>
-      <c r="V7" s="395"/>
-      <c r="W7" s="401"/>
-      <c r="X7" s="384"/>
-      <c r="Y7" s="384"/>
-      <c r="Z7" s="384"/>
-      <c r="AA7" s="384"/>
-      <c r="AB7" s="384"/>
-      <c r="AC7" s="384"/>
-      <c r="AD7" s="384"/>
-      <c r="AE7" s="384"/>
-      <c r="AF7" s="384"/>
-      <c r="AG7" s="384"/>
-      <c r="AH7" s="384"/>
-      <c r="AI7" s="384"/>
-      <c r="AJ7" s="384"/>
-      <c r="AK7" s="394"/>
-      <c r="AL7" s="384"/>
-      <c r="AM7" s="384"/>
-      <c r="AN7" s="384"/>
-      <c r="AO7" s="384"/>
-      <c r="AP7" s="384"/>
-      <c r="AQ7" s="384"/>
-      <c r="AR7" s="384"/>
-      <c r="AS7" s="384"/>
-      <c r="AT7" s="384"/>
-      <c r="AU7" s="384"/>
-      <c r="AV7" s="384"/>
-      <c r="AW7" s="384"/>
-      <c r="AX7" s="384"/>
+      <c r="A7" s="383"/>
+      <c r="B7" s="383"/>
+      <c r="C7" s="383"/>
+      <c r="D7" s="383"/>
+      <c r="E7" s="383"/>
+      <c r="F7" s="383"/>
+      <c r="G7" s="383"/>
+      <c r="H7" s="383"/>
+      <c r="I7" s="383"/>
+      <c r="J7" s="383"/>
+      <c r="K7" s="383"/>
+      <c r="L7" s="383"/>
+      <c r="M7" s="383"/>
+      <c r="N7" s="383"/>
+      <c r="O7" s="383"/>
+      <c r="P7" s="383"/>
+      <c r="Q7" s="383"/>
+      <c r="R7" s="383"/>
+      <c r="S7" s="383"/>
+      <c r="T7" s="383"/>
+      <c r="U7" s="383"/>
+      <c r="V7" s="394"/>
+      <c r="W7" s="400"/>
+      <c r="X7" s="383"/>
+      <c r="Y7" s="383"/>
+      <c r="Z7" s="383"/>
+      <c r="AA7" s="383"/>
+      <c r="AB7" s="383"/>
+      <c r="AC7" s="383"/>
+      <c r="AD7" s="383"/>
+      <c r="AE7" s="383"/>
+      <c r="AF7" s="383"/>
+      <c r="AG7" s="383"/>
+      <c r="AH7" s="383"/>
+      <c r="AI7" s="383"/>
+      <c r="AJ7" s="383"/>
+      <c r="AK7" s="393"/>
+      <c r="AL7" s="383"/>
+      <c r="AM7" s="383"/>
+      <c r="AN7" s="383"/>
+      <c r="AO7" s="383"/>
+      <c r="AP7" s="383"/>
+      <c r="AQ7" s="383"/>
+      <c r="AR7" s="383"/>
+      <c r="AS7" s="383"/>
+      <c r="AT7" s="383"/>
+      <c r="AU7" s="383"/>
+      <c r="AV7" s="383"/>
+      <c r="AW7" s="383"/>
+      <c r="AX7" s="383"/>
       <c r="AY7" s="101" t="s">
         <v>67</v>
       </c>
@@ -12030,124 +12030,124 @@
       <c r="BA7" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="BB7" s="386" t="s">
+      <c r="BB7" s="385" t="s">
         <v>70</v>
       </c>
-      <c r="BC7" s="389" t="s">
+      <c r="BC7" s="388" t="s">
         <v>71</v>
       </c>
-      <c r="BD7" s="389" t="s">
+      <c r="BD7" s="388" t="s">
         <v>72</v>
       </c>
-      <c r="BE7" s="415" t="s">
+      <c r="BE7" s="414" t="s">
         <v>73</v>
       </c>
-      <c r="BF7" s="389" t="s">
+      <c r="BF7" s="388" t="s">
         <v>74</v>
       </c>
-      <c r="BG7" s="389" t="s">
+      <c r="BG7" s="388" t="s">
         <v>75</v>
       </c>
-      <c r="BH7" s="389" t="s">
+      <c r="BH7" s="388" t="s">
         <v>76</v>
       </c>
-      <c r="BI7" s="389" t="s">
+      <c r="BI7" s="388" t="s">
         <v>77</v>
       </c>
-      <c r="BJ7" s="389" t="s">
+      <c r="BJ7" s="388" t="s">
         <v>78</v>
       </c>
-      <c r="BK7" s="389" t="s">
+      <c r="BK7" s="388" t="s">
         <v>79</v>
       </c>
-      <c r="BL7" s="417" t="s">
+      <c r="BL7" s="416" t="s">
         <v>80</v>
       </c>
-      <c r="BM7" s="389" t="s">
+      <c r="BM7" s="388" t="s">
         <v>81</v>
       </c>
-      <c r="BN7" s="386" t="s">
+      <c r="BN7" s="385" t="s">
         <v>82</v>
       </c>
-      <c r="BO7" s="389" t="s">
+      <c r="BO7" s="388" t="s">
         <v>83</v>
       </c>
-      <c r="BP7" s="386" t="s">
+      <c r="BP7" s="385" t="s">
         <v>84</v>
       </c>
-      <c r="BQ7" s="386" t="s">
+      <c r="BQ7" s="385" t="s">
         <v>85</v>
       </c>
-      <c r="BR7" s="384"/>
-      <c r="BS7" s="384"/>
-      <c r="BT7" s="384"/>
-      <c r="BU7" s="394"/>
-      <c r="BW7" s="411"/>
-      <c r="BX7" s="412"/>
-      <c r="BY7" s="413"/>
-      <c r="BZ7" s="413"/>
-      <c r="CA7" s="414"/>
-      <c r="CB7" s="384"/>
-      <c r="CC7" s="384"/>
-      <c r="CD7" s="384"/>
+      <c r="BR7" s="383"/>
+      <c r="BS7" s="383"/>
+      <c r="BT7" s="383"/>
+      <c r="BU7" s="393"/>
+      <c r="BW7" s="410"/>
+      <c r="BX7" s="411"/>
+      <c r="BY7" s="412"/>
+      <c r="BZ7" s="412"/>
+      <c r="CA7" s="413"/>
+      <c r="CB7" s="383"/>
+      <c r="CC7" s="383"/>
+      <c r="CD7" s="383"/>
       <c r="CH7" s="137"/>
       <c r="CI7" s="138"/>
     </row>
     <row r="8" spans="1:87" s="139" customFormat="1" ht="12">
-      <c r="A8" s="385"/>
-      <c r="B8" s="385"/>
-      <c r="C8" s="385"/>
-      <c r="D8" s="385"/>
-      <c r="E8" s="385"/>
-      <c r="F8" s="385"/>
-      <c r="G8" s="385"/>
-      <c r="H8" s="385"/>
-      <c r="I8" s="385"/>
-      <c r="J8" s="385"/>
-      <c r="K8" s="385"/>
-      <c r="L8" s="385"/>
-      <c r="M8" s="385"/>
-      <c r="N8" s="385"/>
-      <c r="O8" s="385"/>
-      <c r="P8" s="385"/>
-      <c r="Q8" s="385"/>
-      <c r="R8" s="385"/>
-      <c r="S8" s="385"/>
-      <c r="T8" s="385"/>
-      <c r="U8" s="385"/>
+      <c r="A8" s="384"/>
+      <c r="B8" s="384"/>
+      <c r="C8" s="384"/>
+      <c r="D8" s="384"/>
+      <c r="E8" s="384"/>
+      <c r="F8" s="384"/>
+      <c r="G8" s="384"/>
+      <c r="H8" s="384"/>
+      <c r="I8" s="384"/>
+      <c r="J8" s="384"/>
+      <c r="K8" s="384"/>
+      <c r="L8" s="384"/>
+      <c r="M8" s="384"/>
+      <c r="N8" s="384"/>
+      <c r="O8" s="384"/>
+      <c r="P8" s="384"/>
+      <c r="Q8" s="384"/>
+      <c r="R8" s="384"/>
+      <c r="S8" s="384"/>
+      <c r="T8" s="384"/>
+      <c r="U8" s="384"/>
       <c r="V8" s="140" t="s">
         <v>86</v>
       </c>
       <c r="W8" s="140" t="s">
         <v>87</v>
       </c>
-      <c r="X8" s="385"/>
-      <c r="Y8" s="385"/>
-      <c r="Z8" s="385"/>
-      <c r="AA8" s="385"/>
-      <c r="AB8" s="385"/>
-      <c r="AC8" s="385"/>
-      <c r="AD8" s="385"/>
-      <c r="AE8" s="385"/>
-      <c r="AF8" s="385"/>
-      <c r="AG8" s="385"/>
-      <c r="AH8" s="385"/>
-      <c r="AI8" s="385"/>
-      <c r="AJ8" s="385"/>
-      <c r="AK8" s="395"/>
-      <c r="AL8" s="385"/>
-      <c r="AM8" s="385"/>
-      <c r="AN8" s="385"/>
-      <c r="AO8" s="385"/>
-      <c r="AP8" s="385"/>
-      <c r="AQ8" s="385"/>
-      <c r="AR8" s="385"/>
-      <c r="AS8" s="385"/>
-      <c r="AT8" s="385"/>
-      <c r="AU8" s="385"/>
-      <c r="AV8" s="385"/>
-      <c r="AW8" s="385"/>
-      <c r="AX8" s="385"/>
+      <c r="X8" s="384"/>
+      <c r="Y8" s="384"/>
+      <c r="Z8" s="384"/>
+      <c r="AA8" s="384"/>
+      <c r="AB8" s="384"/>
+      <c r="AC8" s="384"/>
+      <c r="AD8" s="384"/>
+      <c r="AE8" s="384"/>
+      <c r="AF8" s="384"/>
+      <c r="AG8" s="384"/>
+      <c r="AH8" s="384"/>
+      <c r="AI8" s="384"/>
+      <c r="AJ8" s="384"/>
+      <c r="AK8" s="394"/>
+      <c r="AL8" s="384"/>
+      <c r="AM8" s="384"/>
+      <c r="AN8" s="384"/>
+      <c r="AO8" s="384"/>
+      <c r="AP8" s="384"/>
+      <c r="AQ8" s="384"/>
+      <c r="AR8" s="384"/>
+      <c r="AS8" s="384"/>
+      <c r="AT8" s="384"/>
+      <c r="AU8" s="384"/>
+      <c r="AV8" s="384"/>
+      <c r="AW8" s="384"/>
+      <c r="AX8" s="384"/>
       <c r="AY8" s="102" t="s">
         <v>88</v>
       </c>
@@ -12157,27 +12157,27 @@
       <c r="BA8" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="BB8" s="385"/>
-      <c r="BC8" s="385"/>
-      <c r="BD8" s="385"/>
-      <c r="BE8" s="385"/>
-      <c r="BF8" s="385"/>
-      <c r="BG8" s="385"/>
-      <c r="BH8" s="385"/>
-      <c r="BI8" s="385"/>
-      <c r="BJ8" s="385"/>
-      <c r="BK8" s="385"/>
-      <c r="BL8" s="385"/>
-      <c r="BM8" s="385"/>
-      <c r="BN8" s="385"/>
-      <c r="BO8" s="385"/>
-      <c r="BP8" s="385"/>
-      <c r="BQ8" s="385"/>
-      <c r="BR8" s="385"/>
-      <c r="BS8" s="385"/>
-      <c r="BT8" s="385"/>
-      <c r="BU8" s="395"/>
-      <c r="BW8" s="414"/>
+      <c r="BB8" s="384"/>
+      <c r="BC8" s="384"/>
+      <c r="BD8" s="384"/>
+      <c r="BE8" s="384"/>
+      <c r="BF8" s="384"/>
+      <c r="BG8" s="384"/>
+      <c r="BH8" s="384"/>
+      <c r="BI8" s="384"/>
+      <c r="BJ8" s="384"/>
+      <c r="BK8" s="384"/>
+      <c r="BL8" s="384"/>
+      <c r="BM8" s="384"/>
+      <c r="BN8" s="384"/>
+      <c r="BO8" s="384"/>
+      <c r="BP8" s="384"/>
+      <c r="BQ8" s="384"/>
+      <c r="BR8" s="384"/>
+      <c r="BS8" s="384"/>
+      <c r="BT8" s="384"/>
+      <c r="BU8" s="394"/>
+      <c r="BW8" s="413"/>
       <c r="BX8" s="72" t="s">
         <v>91</v>
       </c>
@@ -12190,9 +12190,9 @@
       <c r="CA8" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="CB8" s="406"/>
-      <c r="CC8" s="406"/>
-      <c r="CD8" s="406"/>
+      <c r="CB8" s="405"/>
+      <c r="CC8" s="405"/>
+      <c r="CD8" s="405"/>
       <c r="CE8" s="136"/>
       <c r="CF8" s="141"/>
       <c r="CH8" s="137"/>
@@ -14959,88 +14959,88 @@
       <c r="CD2" s="12"/>
     </row>
     <row r="3" spans="1:87" s="16" customFormat="1" ht="24" customHeight="1" outlineLevel="1">
-      <c r="A3" s="431"/>
-      <c r="B3" s="430"/>
-      <c r="C3" s="430"/>
-      <c r="D3" s="430"/>
-      <c r="E3" s="430"/>
-      <c r="F3" s="430"/>
-      <c r="G3" s="430"/>
-      <c r="H3" s="430"/>
-      <c r="I3" s="430"/>
-      <c r="J3" s="430"/>
-      <c r="K3" s="430"/>
-      <c r="L3" s="430"/>
-      <c r="M3" s="430"/>
-      <c r="N3" s="430"/>
-      <c r="O3" s="430"/>
-      <c r="P3" s="430"/>
-      <c r="Q3" s="430"/>
-      <c r="R3" s="430"/>
-      <c r="S3" s="430"/>
-      <c r="T3" s="430"/>
-      <c r="U3" s="430"/>
-      <c r="V3" s="430"/>
-      <c r="W3" s="430"/>
-      <c r="X3" s="430"/>
-      <c r="Y3" s="430"/>
-      <c r="Z3" s="430"/>
-      <c r="AA3" s="430"/>
-      <c r="AB3" s="430"/>
-      <c r="AC3" s="430"/>
-      <c r="AD3" s="430"/>
-      <c r="AE3" s="430"/>
-      <c r="AF3" s="430"/>
-      <c r="AG3" s="430"/>
-      <c r="AH3" s="430"/>
-      <c r="AI3" s="430"/>
-      <c r="AJ3" s="430"/>
-      <c r="AK3" s="430"/>
-      <c r="AL3" s="430"/>
-      <c r="AM3" s="430"/>
-      <c r="AN3" s="430"/>
-      <c r="AO3" s="430"/>
-      <c r="AP3" s="430"/>
-      <c r="AQ3" s="430"/>
-      <c r="AR3" s="430"/>
-      <c r="AS3" s="430"/>
-      <c r="AT3" s="430"/>
-      <c r="AU3" s="430"/>
-      <c r="AV3" s="430"/>
-      <c r="AW3" s="430"/>
-      <c r="AX3" s="430"/>
-      <c r="AY3" s="430"/>
-      <c r="AZ3" s="430"/>
-      <c r="BA3" s="430"/>
-      <c r="BB3" s="430"/>
-      <c r="BC3" s="430"/>
-      <c r="BD3" s="430"/>
-      <c r="BE3" s="430"/>
-      <c r="BF3" s="430"/>
-      <c r="BG3" s="430"/>
-      <c r="BH3" s="430"/>
-      <c r="BI3" s="430"/>
-      <c r="BJ3" s="430"/>
-      <c r="BK3" s="430"/>
-      <c r="BL3" s="430"/>
-      <c r="BM3" s="430"/>
-      <c r="BN3" s="430"/>
-      <c r="BO3" s="430"/>
-      <c r="BP3" s="430"/>
-      <c r="BQ3" s="430"/>
-      <c r="BR3" s="430"/>
-      <c r="BS3" s="430"/>
-      <c r="BT3" s="430"/>
-      <c r="BU3" s="430"/>
+      <c r="A3" s="430"/>
+      <c r="B3" s="429"/>
+      <c r="C3" s="429"/>
+      <c r="D3" s="429"/>
+      <c r="E3" s="429"/>
+      <c r="F3" s="429"/>
+      <c r="G3" s="429"/>
+      <c r="H3" s="429"/>
+      <c r="I3" s="429"/>
+      <c r="J3" s="429"/>
+      <c r="K3" s="429"/>
+      <c r="L3" s="429"/>
+      <c r="M3" s="429"/>
+      <c r="N3" s="429"/>
+      <c r="O3" s="429"/>
+      <c r="P3" s="429"/>
+      <c r="Q3" s="429"/>
+      <c r="R3" s="429"/>
+      <c r="S3" s="429"/>
+      <c r="T3" s="429"/>
+      <c r="U3" s="429"/>
+      <c r="V3" s="429"/>
+      <c r="W3" s="429"/>
+      <c r="X3" s="429"/>
+      <c r="Y3" s="429"/>
+      <c r="Z3" s="429"/>
+      <c r="AA3" s="429"/>
+      <c r="AB3" s="429"/>
+      <c r="AC3" s="429"/>
+      <c r="AD3" s="429"/>
+      <c r="AE3" s="429"/>
+      <c r="AF3" s="429"/>
+      <c r="AG3" s="429"/>
+      <c r="AH3" s="429"/>
+      <c r="AI3" s="429"/>
+      <c r="AJ3" s="429"/>
+      <c r="AK3" s="429"/>
+      <c r="AL3" s="429"/>
+      <c r="AM3" s="429"/>
+      <c r="AN3" s="429"/>
+      <c r="AO3" s="429"/>
+      <c r="AP3" s="429"/>
+      <c r="AQ3" s="429"/>
+      <c r="AR3" s="429"/>
+      <c r="AS3" s="429"/>
+      <c r="AT3" s="429"/>
+      <c r="AU3" s="429"/>
+      <c r="AV3" s="429"/>
+      <c r="AW3" s="429"/>
+      <c r="AX3" s="429"/>
+      <c r="AY3" s="429"/>
+      <c r="AZ3" s="429"/>
+      <c r="BA3" s="429"/>
+      <c r="BB3" s="429"/>
+      <c r="BC3" s="429"/>
+      <c r="BD3" s="429"/>
+      <c r="BE3" s="429"/>
+      <c r="BF3" s="429"/>
+      <c r="BG3" s="429"/>
+      <c r="BH3" s="429"/>
+      <c r="BI3" s="429"/>
+      <c r="BJ3" s="429"/>
+      <c r="BK3" s="429"/>
+      <c r="BL3" s="429"/>
+      <c r="BM3" s="429"/>
+      <c r="BN3" s="429"/>
+      <c r="BO3" s="429"/>
+      <c r="BP3" s="429"/>
+      <c r="BQ3" s="429"/>
+      <c r="BR3" s="429"/>
+      <c r="BS3" s="429"/>
+      <c r="BT3" s="429"/>
+      <c r="BU3" s="429"/>
       <c r="BV3" s="110"/>
-      <c r="BW3" s="429" t="s">
+      <c r="BW3" s="428" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="430"/>
-      <c r="BY3" s="430"/>
-      <c r="BZ3" s="430"/>
-      <c r="CA3" s="430"/>
-      <c r="CB3" s="430"/>
+      <c r="BX3" s="429"/>
+      <c r="BY3" s="429"/>
+      <c r="BZ3" s="429"/>
+      <c r="CA3" s="429"/>
+      <c r="CB3" s="429"/>
       <c r="CC3" s="71"/>
       <c r="CD3" s="71"/>
       <c r="CE3" s="16" t="s">
@@ -15124,12 +15124,12 @@
       <c r="BT4" s="15"/>
       <c r="BU4" s="15"/>
       <c r="BV4" s="111"/>
-      <c r="BW4" s="430"/>
-      <c r="BX4" s="430"/>
-      <c r="BY4" s="430"/>
-      <c r="BZ4" s="430"/>
-      <c r="CA4" s="430"/>
-      <c r="CB4" s="430"/>
+      <c r="BW4" s="429"/>
+      <c r="BX4" s="429"/>
+      <c r="BY4" s="429"/>
+      <c r="BZ4" s="429"/>
+      <c r="CA4" s="429"/>
+      <c r="CB4" s="429"/>
       <c r="CC4" s="71"/>
       <c r="CD4" s="71"/>
     </row>
@@ -15207,12 +15207,12 @@
       <c r="BT5" s="15"/>
       <c r="BU5" s="15"/>
       <c r="BV5" s="111"/>
-      <c r="BW5" s="363"/>
-      <c r="BX5" s="363"/>
-      <c r="BY5" s="363"/>
-      <c r="BZ5" s="363"/>
-      <c r="CA5" s="363"/>
-      <c r="CB5" s="363"/>
+      <c r="BW5" s="362"/>
+      <c r="BX5" s="362"/>
+      <c r="BY5" s="362"/>
+      <c r="BZ5" s="362"/>
+      <c r="CA5" s="362"/>
+      <c r="CB5" s="362"/>
       <c r="CC5" s="71"/>
       <c r="CD5" s="71"/>
     </row>
@@ -15290,12 +15290,12 @@
       <c r="BT6" s="18"/>
       <c r="BU6" s="18"/>
       <c r="BV6" s="112"/>
-      <c r="BW6" s="363"/>
-      <c r="BX6" s="363"/>
-      <c r="BY6" s="363"/>
-      <c r="BZ6" s="363"/>
-      <c r="CA6" s="363"/>
-      <c r="CB6" s="363"/>
+      <c r="BW6" s="362"/>
+      <c r="BX6" s="362"/>
+      <c r="BY6" s="362"/>
+      <c r="BZ6" s="362"/>
+      <c r="CA6" s="362"/>
+      <c r="CB6" s="362"/>
       <c r="CC6" s="71"/>
       <c r="CD6" s="71"/>
     </row>
@@ -15383,358 +15383,358 @@
       <c r="CD7" s="25"/>
     </row>
     <row r="8" spans="1:87" s="11" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A8" s="392" t="s">
+      <c r="A8" s="391" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="402" t="s">
+      <c r="B8" s="401" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="390" t="s">
+      <c r="C8" s="389" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="398" t="s">
+      <c r="D8" s="397" t="s">
         <v>141</v>
       </c>
-      <c r="E8" s="398" t="s">
+      <c r="E8" s="397" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="427" t="s">
+      <c r="F8" s="426" t="s">
         <v>142</v>
       </c>
-      <c r="G8" s="424" t="s">
+      <c r="G8" s="423" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="369" t="s">
+      <c r="H8" s="368" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="369" t="s">
+      <c r="I8" s="368" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="424" t="s">
+      <c r="J8" s="423" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="428" t="s">
+      <c r="K8" s="427" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="387"/>
-      <c r="M8" s="387"/>
-      <c r="N8" s="387"/>
-      <c r="O8" s="387"/>
-      <c r="P8" s="387"/>
-      <c r="Q8" s="387"/>
-      <c r="R8" s="387"/>
-      <c r="S8" s="387"/>
-      <c r="T8" s="387"/>
-      <c r="U8" s="387"/>
-      <c r="V8" s="387"/>
-      <c r="W8" s="387"/>
-      <c r="X8" s="387"/>
-      <c r="Y8" s="424" t="s">
+      <c r="L8" s="386"/>
+      <c r="M8" s="386"/>
+      <c r="N8" s="386"/>
+      <c r="O8" s="386"/>
+      <c r="P8" s="386"/>
+      <c r="Q8" s="386"/>
+      <c r="R8" s="386"/>
+      <c r="S8" s="386"/>
+      <c r="T8" s="386"/>
+      <c r="U8" s="386"/>
+      <c r="V8" s="386"/>
+      <c r="W8" s="386"/>
+      <c r="X8" s="386"/>
+      <c r="Y8" s="423" t="s">
         <v>15</v>
       </c>
-      <c r="Z8" s="387"/>
-      <c r="AA8" s="387"/>
-      <c r="AB8" s="387"/>
-      <c r="AC8" s="387"/>
-      <c r="AD8" s="387"/>
-      <c r="AE8" s="387"/>
-      <c r="AF8" s="387"/>
-      <c r="AG8" s="387"/>
-      <c r="AH8" s="387"/>
-      <c r="AI8" s="387"/>
-      <c r="AJ8" s="387"/>
-      <c r="AK8" s="387"/>
-      <c r="AL8" s="387"/>
-      <c r="AM8" s="387"/>
-      <c r="AN8" s="387"/>
-      <c r="AO8" s="388"/>
-      <c r="AP8" s="424" t="s">
+      <c r="Z8" s="386"/>
+      <c r="AA8" s="386"/>
+      <c r="AB8" s="386"/>
+      <c r="AC8" s="386"/>
+      <c r="AD8" s="386"/>
+      <c r="AE8" s="386"/>
+      <c r="AF8" s="386"/>
+      <c r="AG8" s="386"/>
+      <c r="AH8" s="386"/>
+      <c r="AI8" s="386"/>
+      <c r="AJ8" s="386"/>
+      <c r="AK8" s="386"/>
+      <c r="AL8" s="386"/>
+      <c r="AM8" s="386"/>
+      <c r="AN8" s="386"/>
+      <c r="AO8" s="387"/>
+      <c r="AP8" s="423" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="424" t="s">
+      <c r="AQ8" s="423" t="s">
         <v>17</v>
       </c>
-      <c r="AR8" s="424" t="s">
+      <c r="AR8" s="423" t="s">
         <v>18</v>
       </c>
-      <c r="AS8" s="424" t="s">
+      <c r="AS8" s="423" t="s">
         <v>19</v>
       </c>
-      <c r="AT8" s="424" t="s">
+      <c r="AT8" s="423" t="s">
         <v>20</v>
       </c>
-      <c r="AU8" s="424" t="s">
+      <c r="AU8" s="423" t="s">
         <v>21</v>
       </c>
-      <c r="AV8" s="390" t="s">
+      <c r="AV8" s="389" t="s">
         <v>22</v>
       </c>
-      <c r="AW8" s="390" t="s">
+      <c r="AW8" s="389" t="s">
         <v>23</v>
       </c>
-      <c r="AX8" s="390" t="s">
+      <c r="AX8" s="389" t="s">
         <v>24</v>
       </c>
-      <c r="AY8" s="386" t="s">
+      <c r="AY8" s="385" t="s">
         <v>25</v>
       </c>
-      <c r="AZ8" s="387"/>
-      <c r="BA8" s="387"/>
-      <c r="BB8" s="387"/>
-      <c r="BC8" s="387"/>
-      <c r="BD8" s="387"/>
-      <c r="BE8" s="387"/>
-      <c r="BF8" s="387"/>
-      <c r="BG8" s="387"/>
-      <c r="BH8" s="387"/>
-      <c r="BI8" s="387"/>
-      <c r="BJ8" s="387"/>
-      <c r="BK8" s="387"/>
-      <c r="BL8" s="387"/>
-      <c r="BM8" s="387"/>
-      <c r="BN8" s="387"/>
-      <c r="BO8" s="387"/>
-      <c r="BP8" s="388"/>
-      <c r="BQ8" s="407" t="s">
+      <c r="AZ8" s="386"/>
+      <c r="BA8" s="386"/>
+      <c r="BB8" s="386"/>
+      <c r="BC8" s="386"/>
+      <c r="BD8" s="386"/>
+      <c r="BE8" s="386"/>
+      <c r="BF8" s="386"/>
+      <c r="BG8" s="386"/>
+      <c r="BH8" s="386"/>
+      <c r="BI8" s="386"/>
+      <c r="BJ8" s="386"/>
+      <c r="BK8" s="386"/>
+      <c r="BL8" s="386"/>
+      <c r="BM8" s="386"/>
+      <c r="BN8" s="386"/>
+      <c r="BO8" s="386"/>
+      <c r="BP8" s="387"/>
+      <c r="BQ8" s="406" t="s">
         <v>26</v>
       </c>
-      <c r="BR8" s="400"/>
-      <c r="BS8" s="386" t="s">
+      <c r="BR8" s="399"/>
+      <c r="BS8" s="385" t="s">
         <v>143</v>
       </c>
-      <c r="BT8" s="386" t="s">
+      <c r="BT8" s="385" t="s">
         <v>27</v>
       </c>
-      <c r="BU8" s="418" t="s">
+      <c r="BU8" s="417" t="s">
         <v>28</v>
       </c>
       <c r="BV8" s="114"/>
-      <c r="BW8" s="419" t="s">
+      <c r="BW8" s="418" t="s">
         <v>29</v>
       </c>
-      <c r="BX8" s="408" t="s">
+      <c r="BX8" s="407" t="s">
         <v>30</v>
       </c>
-      <c r="BY8" s="409"/>
-      <c r="BZ8" s="409"/>
-      <c r="CA8" s="400"/>
-      <c r="CB8" s="420" t="s">
+      <c r="BY8" s="408"/>
+      <c r="BZ8" s="408"/>
+      <c r="CA8" s="399"/>
+      <c r="CB8" s="419" t="s">
         <v>31</v>
       </c>
-      <c r="CC8" s="405" t="s">
+      <c r="CC8" s="404" t="s">
         <v>32</v>
       </c>
-      <c r="CD8" s="405" t="s">
+      <c r="CD8" s="404" t="s">
         <v>33</v>
       </c>
       <c r="CH8" s="27"/>
       <c r="CI8" s="28"/>
     </row>
     <row r="9" spans="1:87" s="11" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A9" s="384"/>
-      <c r="B9" s="384"/>
-      <c r="C9" s="384"/>
-      <c r="D9" s="384"/>
-      <c r="E9" s="384"/>
-      <c r="F9" s="384"/>
-      <c r="G9" s="384"/>
-      <c r="H9" s="384"/>
-      <c r="I9" s="384"/>
-      <c r="J9" s="384"/>
-      <c r="K9" s="421" t="s">
+      <c r="A9" s="383"/>
+      <c r="B9" s="383"/>
+      <c r="C9" s="383"/>
+      <c r="D9" s="383"/>
+      <c r="E9" s="383"/>
+      <c r="F9" s="383"/>
+      <c r="G9" s="383"/>
+      <c r="H9" s="383"/>
+      <c r="I9" s="383"/>
+      <c r="J9" s="383"/>
+      <c r="K9" s="420" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="421" t="s">
+      <c r="L9" s="420" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="421" t="s">
+      <c r="M9" s="420" t="s">
         <v>36</v>
       </c>
-      <c r="N9" s="421" t="s">
+      <c r="N9" s="420" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="421" t="s">
+      <c r="O9" s="420" t="s">
         <v>38</v>
       </c>
-      <c r="P9" s="421" t="s">
+      <c r="P9" s="420" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="421" t="s">
+      <c r="Q9" s="420" t="s">
         <v>40</v>
       </c>
-      <c r="R9" s="421" t="s">
+      <c r="R9" s="420" t="s">
         <v>41</v>
       </c>
-      <c r="S9" s="421" t="s">
+      <c r="S9" s="420" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="421" t="s">
+      <c r="T9" s="420" t="s">
         <v>43</v>
       </c>
-      <c r="U9" s="421" t="s">
+      <c r="U9" s="420" t="s">
         <v>44</v>
       </c>
-      <c r="V9" s="433" t="s">
+      <c r="V9" s="432" t="s">
         <v>45</v>
       </c>
-      <c r="W9" s="400"/>
-      <c r="X9" s="421" t="s">
+      <c r="W9" s="399"/>
+      <c r="X9" s="420" t="s">
         <v>46</v>
       </c>
-      <c r="Y9" s="423" t="s">
+      <c r="Y9" s="422" t="s">
         <v>47</v>
       </c>
-      <c r="Z9" s="423" t="s">
+      <c r="Z9" s="422" t="s">
         <v>48</v>
       </c>
-      <c r="AA9" s="423" t="s">
+      <c r="AA9" s="422" t="s">
         <v>49</v>
       </c>
-      <c r="AB9" s="423" t="s">
+      <c r="AB9" s="422" t="s">
         <v>50</v>
       </c>
-      <c r="AC9" s="331" t="s">
+      <c r="AC9" s="330" t="s">
         <v>51</v>
       </c>
-      <c r="AD9" s="331" t="s">
+      <c r="AD9" s="330" t="s">
         <v>144</v>
       </c>
-      <c r="AE9" s="331" t="s">
+      <c r="AE9" s="330" t="s">
         <v>53</v>
       </c>
-      <c r="AF9" s="331" t="s">
+      <c r="AF9" s="330" t="s">
         <v>54</v>
       </c>
-      <c r="AG9" s="423" t="s">
+      <c r="AG9" s="422" t="s">
         <v>55</v>
       </c>
-      <c r="AH9" s="331" t="s">
+      <c r="AH9" s="330" t="s">
         <v>56</v>
       </c>
-      <c r="AI9" s="331" t="s">
+      <c r="AI9" s="330" t="s">
         <v>57</v>
       </c>
-      <c r="AJ9" s="423" t="s">
+      <c r="AJ9" s="422" t="s">
         <v>58</v>
       </c>
-      <c r="AK9" s="393" t="s">
+      <c r="AK9" s="392" t="s">
         <v>59</v>
       </c>
-      <c r="AL9" s="390" t="s">
+      <c r="AL9" s="389" t="s">
         <v>60</v>
       </c>
-      <c r="AM9" s="423" t="s">
+      <c r="AM9" s="422" t="s">
         <v>61</v>
       </c>
-      <c r="AN9" s="397" t="s">
+      <c r="AN9" s="396" t="s">
         <v>62</v>
       </c>
-      <c r="AO9" s="390" t="s">
+      <c r="AO9" s="389" t="s">
         <v>63</v>
       </c>
-      <c r="AP9" s="384"/>
-      <c r="AQ9" s="384"/>
-      <c r="AR9" s="384"/>
-      <c r="AS9" s="384"/>
-      <c r="AT9" s="384"/>
-      <c r="AU9" s="384"/>
-      <c r="AV9" s="384"/>
-      <c r="AW9" s="384"/>
-      <c r="AX9" s="384"/>
-      <c r="AY9" s="386" t="s">
+      <c r="AP9" s="383"/>
+      <c r="AQ9" s="383"/>
+      <c r="AR9" s="383"/>
+      <c r="AS9" s="383"/>
+      <c r="AT9" s="383"/>
+      <c r="AU9" s="383"/>
+      <c r="AV9" s="383"/>
+      <c r="AW9" s="383"/>
+      <c r="AX9" s="383"/>
+      <c r="AY9" s="385" t="s">
         <v>25</v>
       </c>
-      <c r="AZ9" s="387"/>
-      <c r="BA9" s="387"/>
-      <c r="BB9" s="387"/>
-      <c r="BC9" s="387"/>
-      <c r="BD9" s="387"/>
-      <c r="BE9" s="387"/>
-      <c r="BF9" s="387"/>
-      <c r="BG9" s="387"/>
-      <c r="BH9" s="387"/>
-      <c r="BI9" s="387"/>
-      <c r="BJ9" s="388"/>
-      <c r="BK9" s="386" t="s">
+      <c r="AZ9" s="386"/>
+      <c r="BA9" s="386"/>
+      <c r="BB9" s="386"/>
+      <c r="BC9" s="386"/>
+      <c r="BD9" s="386"/>
+      <c r="BE9" s="386"/>
+      <c r="BF9" s="386"/>
+      <c r="BG9" s="386"/>
+      <c r="BH9" s="386"/>
+      <c r="BI9" s="386"/>
+      <c r="BJ9" s="387"/>
+      <c r="BK9" s="385" t="s">
         <v>64</v>
       </c>
-      <c r="BL9" s="387"/>
-      <c r="BM9" s="387"/>
-      <c r="BN9" s="387"/>
-      <c r="BO9" s="387"/>
-      <c r="BP9" s="388"/>
-      <c r="BQ9" s="383" t="s">
+      <c r="BL9" s="386"/>
+      <c r="BM9" s="386"/>
+      <c r="BN9" s="386"/>
+      <c r="BO9" s="386"/>
+      <c r="BP9" s="387"/>
+      <c r="BQ9" s="382" t="s">
         <v>65</v>
       </c>
-      <c r="BR9" s="383" t="s">
+      <c r="BR9" s="382" t="s">
         <v>66</v>
       </c>
-      <c r="BS9" s="384"/>
-      <c r="BT9" s="384"/>
-      <c r="BU9" s="394"/>
+      <c r="BS9" s="383"/>
+      <c r="BT9" s="383"/>
+      <c r="BU9" s="393"/>
       <c r="BV9" s="114"/>
-      <c r="BW9" s="411"/>
-      <c r="BX9" s="394"/>
-      <c r="BY9" s="425"/>
-      <c r="BZ9" s="425"/>
-      <c r="CA9" s="411"/>
-      <c r="CB9" s="384"/>
-      <c r="CC9" s="384"/>
-      <c r="CD9" s="384"/>
+      <c r="BW9" s="410"/>
+      <c r="BX9" s="393"/>
+      <c r="BY9" s="424"/>
+      <c r="BZ9" s="424"/>
+      <c r="CA9" s="410"/>
+      <c r="CB9" s="383"/>
+      <c r="CC9" s="383"/>
+      <c r="CD9" s="383"/>
       <c r="CH9" s="27"/>
       <c r="CI9" s="28"/>
     </row>
     <row r="10" spans="1:87" s="29" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A10" s="384"/>
-      <c r="B10" s="384"/>
-      <c r="C10" s="384"/>
-      <c r="D10" s="384"/>
-      <c r="E10" s="384"/>
-      <c r="F10" s="384"/>
-      <c r="G10" s="384"/>
-      <c r="H10" s="384"/>
-      <c r="I10" s="384"/>
-      <c r="J10" s="384"/>
-      <c r="K10" s="384"/>
-      <c r="L10" s="384"/>
-      <c r="M10" s="384"/>
-      <c r="N10" s="384"/>
-      <c r="O10" s="384"/>
-      <c r="P10" s="384"/>
-      <c r="Q10" s="384"/>
-      <c r="R10" s="384"/>
-      <c r="S10" s="384"/>
-      <c r="T10" s="384"/>
-      <c r="U10" s="384"/>
-      <c r="V10" s="395"/>
-      <c r="W10" s="401"/>
-      <c r="X10" s="384"/>
-      <c r="Y10" s="384"/>
-      <c r="Z10" s="384"/>
-      <c r="AA10" s="384"/>
-      <c r="AB10" s="384"/>
-      <c r="AC10" s="384"/>
-      <c r="AD10" s="384"/>
-      <c r="AE10" s="384"/>
-      <c r="AF10" s="384"/>
-      <c r="AG10" s="384"/>
-      <c r="AH10" s="384"/>
-      <c r="AI10" s="384"/>
-      <c r="AJ10" s="384"/>
-      <c r="AK10" s="394"/>
-      <c r="AL10" s="384"/>
-      <c r="AM10" s="384"/>
-      <c r="AN10" s="384"/>
-      <c r="AO10" s="384"/>
-      <c r="AP10" s="384"/>
-      <c r="AQ10" s="384"/>
-      <c r="AR10" s="384"/>
-      <c r="AS10" s="384"/>
-      <c r="AT10" s="384"/>
-      <c r="AU10" s="384"/>
-      <c r="AV10" s="384"/>
-      <c r="AW10" s="384"/>
-      <c r="AX10" s="384"/>
+      <c r="A10" s="383"/>
+      <c r="B10" s="383"/>
+      <c r="C10" s="383"/>
+      <c r="D10" s="383"/>
+      <c r="E10" s="383"/>
+      <c r="F10" s="383"/>
+      <c r="G10" s="383"/>
+      <c r="H10" s="383"/>
+      <c r="I10" s="383"/>
+      <c r="J10" s="383"/>
+      <c r="K10" s="383"/>
+      <c r="L10" s="383"/>
+      <c r="M10" s="383"/>
+      <c r="N10" s="383"/>
+      <c r="O10" s="383"/>
+      <c r="P10" s="383"/>
+      <c r="Q10" s="383"/>
+      <c r="R10" s="383"/>
+      <c r="S10" s="383"/>
+      <c r="T10" s="383"/>
+      <c r="U10" s="383"/>
+      <c r="V10" s="394"/>
+      <c r="W10" s="400"/>
+      <c r="X10" s="383"/>
+      <c r="Y10" s="383"/>
+      <c r="Z10" s="383"/>
+      <c r="AA10" s="383"/>
+      <c r="AB10" s="383"/>
+      <c r="AC10" s="383"/>
+      <c r="AD10" s="383"/>
+      <c r="AE10" s="383"/>
+      <c r="AF10" s="383"/>
+      <c r="AG10" s="383"/>
+      <c r="AH10" s="383"/>
+      <c r="AI10" s="383"/>
+      <c r="AJ10" s="383"/>
+      <c r="AK10" s="393"/>
+      <c r="AL10" s="383"/>
+      <c r="AM10" s="383"/>
+      <c r="AN10" s="383"/>
+      <c r="AO10" s="383"/>
+      <c r="AP10" s="383"/>
+      <c r="AQ10" s="383"/>
+      <c r="AR10" s="383"/>
+      <c r="AS10" s="383"/>
+      <c r="AT10" s="383"/>
+      <c r="AU10" s="383"/>
+      <c r="AV10" s="383"/>
+      <c r="AW10" s="383"/>
+      <c r="AX10" s="383"/>
       <c r="AY10" s="101" t="s">
         <v>67</v>
       </c>
@@ -15744,123 +15744,123 @@
       <c r="BA10" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="BB10" s="432" t="s">
+      <c r="BB10" s="431" t="s">
         <v>70</v>
       </c>
-      <c r="BC10" s="422" t="s">
+      <c r="BC10" s="421" t="s">
         <v>71</v>
       </c>
-      <c r="BD10" s="422" t="s">
+      <c r="BD10" s="421" t="s">
         <v>72</v>
       </c>
-      <c r="BE10" s="422" t="s">
+      <c r="BE10" s="421" t="s">
         <v>145</v>
       </c>
-      <c r="BF10" s="422" t="s">
+      <c r="BF10" s="421" t="s">
         <v>74</v>
       </c>
-      <c r="BG10" s="422" t="s">
+      <c r="BG10" s="421" t="s">
         <v>75</v>
       </c>
-      <c r="BH10" s="422" t="s">
+      <c r="BH10" s="421" t="s">
         <v>76</v>
       </c>
-      <c r="BI10" s="422" t="s">
+      <c r="BI10" s="421" t="s">
         <v>79</v>
       </c>
-      <c r="BJ10" s="434" t="s">
+      <c r="BJ10" s="433" t="s">
         <v>80</v>
       </c>
-      <c r="BK10" s="422" t="s">
+      <c r="BK10" s="421" t="s">
         <v>81</v>
       </c>
-      <c r="BL10" s="426" t="s">
+      <c r="BL10" s="425" t="s">
         <v>82</v>
       </c>
-      <c r="BM10" s="422" t="s">
+      <c r="BM10" s="421" t="s">
         <v>83</v>
       </c>
-      <c r="BN10" s="426" t="s">
+      <c r="BN10" s="425" t="s">
         <v>84</v>
       </c>
-      <c r="BO10" s="426" t="s">
+      <c r="BO10" s="425" t="s">
         <v>146</v>
       </c>
-      <c r="BP10" s="386" t="s">
+      <c r="BP10" s="385" t="s">
         <v>85</v>
       </c>
-      <c r="BQ10" s="384"/>
-      <c r="BR10" s="384"/>
-      <c r="BS10" s="384"/>
-      <c r="BT10" s="384"/>
-      <c r="BU10" s="394"/>
+      <c r="BQ10" s="383"/>
+      <c r="BR10" s="383"/>
+      <c r="BS10" s="383"/>
+      <c r="BT10" s="383"/>
+      <c r="BU10" s="393"/>
       <c r="BV10" s="114"/>
-      <c r="BW10" s="411"/>
-      <c r="BX10" s="412"/>
-      <c r="BY10" s="413"/>
-      <c r="BZ10" s="413"/>
-      <c r="CA10" s="414"/>
-      <c r="CB10" s="384"/>
-      <c r="CC10" s="384"/>
-      <c r="CD10" s="384"/>
+      <c r="BW10" s="410"/>
+      <c r="BX10" s="411"/>
+      <c r="BY10" s="412"/>
+      <c r="BZ10" s="412"/>
+      <c r="CA10" s="413"/>
+      <c r="CB10" s="383"/>
+      <c r="CC10" s="383"/>
+      <c r="CD10" s="383"/>
       <c r="CH10" s="27"/>
       <c r="CI10" s="28"/>
     </row>
     <row r="11" spans="1:87" s="29" customFormat="1" ht="38.25" customHeight="1">
-      <c r="A11" s="385"/>
-      <c r="B11" s="385"/>
-      <c r="C11" s="385"/>
-      <c r="D11" s="385"/>
-      <c r="E11" s="385"/>
-      <c r="F11" s="385"/>
-      <c r="G11" s="385"/>
-      <c r="H11" s="385"/>
-      <c r="I11" s="385"/>
-      <c r="J11" s="385"/>
-      <c r="K11" s="385"/>
-      <c r="L11" s="385"/>
-      <c r="M11" s="385"/>
-      <c r="N11" s="385"/>
-      <c r="O11" s="385"/>
-      <c r="P11" s="385"/>
-      <c r="Q11" s="385"/>
-      <c r="R11" s="385"/>
-      <c r="S11" s="385"/>
-      <c r="T11" s="385"/>
-      <c r="U11" s="385"/>
+      <c r="A11" s="384"/>
+      <c r="B11" s="384"/>
+      <c r="C11" s="384"/>
+      <c r="D11" s="384"/>
+      <c r="E11" s="384"/>
+      <c r="F11" s="384"/>
+      <c r="G11" s="384"/>
+      <c r="H11" s="384"/>
+      <c r="I11" s="384"/>
+      <c r="J11" s="384"/>
+      <c r="K11" s="384"/>
+      <c r="L11" s="384"/>
+      <c r="M11" s="384"/>
+      <c r="N11" s="384"/>
+      <c r="O11" s="384"/>
+      <c r="P11" s="384"/>
+      <c r="Q11" s="384"/>
+      <c r="R11" s="384"/>
+      <c r="S11" s="384"/>
+      <c r="T11" s="384"/>
+      <c r="U11" s="384"/>
       <c r="V11" s="30" t="s">
         <v>86</v>
       </c>
       <c r="W11" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="X11" s="385"/>
-      <c r="Y11" s="385"/>
-      <c r="Z11" s="385"/>
-      <c r="AA11" s="385"/>
-      <c r="AB11" s="385"/>
-      <c r="AC11" s="385"/>
-      <c r="AD11" s="385"/>
-      <c r="AE11" s="385"/>
-      <c r="AF11" s="385"/>
-      <c r="AG11" s="385"/>
-      <c r="AH11" s="385"/>
-      <c r="AI11" s="385"/>
-      <c r="AJ11" s="385"/>
-      <c r="AK11" s="395"/>
-      <c r="AL11" s="385"/>
-      <c r="AM11" s="385"/>
-      <c r="AN11" s="385"/>
-      <c r="AO11" s="385"/>
-      <c r="AP11" s="385"/>
-      <c r="AQ11" s="385"/>
-      <c r="AR11" s="385"/>
-      <c r="AS11" s="385"/>
-      <c r="AT11" s="385"/>
-      <c r="AU11" s="385"/>
-      <c r="AV11" s="385"/>
-      <c r="AW11" s="385"/>
-      <c r="AX11" s="385"/>
+      <c r="X11" s="384"/>
+      <c r="Y11" s="384"/>
+      <c r="Z11" s="384"/>
+      <c r="AA11" s="384"/>
+      <c r="AB11" s="384"/>
+      <c r="AC11" s="384"/>
+      <c r="AD11" s="384"/>
+      <c r="AE11" s="384"/>
+      <c r="AF11" s="384"/>
+      <c r="AG11" s="384"/>
+      <c r="AH11" s="384"/>
+      <c r="AI11" s="384"/>
+      <c r="AJ11" s="384"/>
+      <c r="AK11" s="394"/>
+      <c r="AL11" s="384"/>
+      <c r="AM11" s="384"/>
+      <c r="AN11" s="384"/>
+      <c r="AO11" s="384"/>
+      <c r="AP11" s="384"/>
+      <c r="AQ11" s="384"/>
+      <c r="AR11" s="384"/>
+      <c r="AS11" s="384"/>
+      <c r="AT11" s="384"/>
+      <c r="AU11" s="384"/>
+      <c r="AV11" s="384"/>
+      <c r="AW11" s="384"/>
+      <c r="AX11" s="384"/>
       <c r="AY11" s="102" t="s">
         <v>88</v>
       </c>
@@ -15870,28 +15870,28 @@
       <c r="BA11" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="BB11" s="385"/>
-      <c r="BC11" s="385"/>
-      <c r="BD11" s="385"/>
-      <c r="BE11" s="385"/>
-      <c r="BF11" s="385"/>
-      <c r="BG11" s="385"/>
-      <c r="BH11" s="385"/>
-      <c r="BI11" s="385"/>
-      <c r="BJ11" s="385"/>
-      <c r="BK11" s="385"/>
-      <c r="BL11" s="385"/>
-      <c r="BM11" s="385"/>
-      <c r="BN11" s="385"/>
-      <c r="BO11" s="385"/>
-      <c r="BP11" s="385"/>
-      <c r="BQ11" s="385"/>
-      <c r="BR11" s="385"/>
-      <c r="BS11" s="385"/>
-      <c r="BT11" s="385"/>
-      <c r="BU11" s="395"/>
+      <c r="BB11" s="384"/>
+      <c r="BC11" s="384"/>
+      <c r="BD11" s="384"/>
+      <c r="BE11" s="384"/>
+      <c r="BF11" s="384"/>
+      <c r="BG11" s="384"/>
+      <c r="BH11" s="384"/>
+      <c r="BI11" s="384"/>
+      <c r="BJ11" s="384"/>
+      <c r="BK11" s="384"/>
+      <c r="BL11" s="384"/>
+      <c r="BM11" s="384"/>
+      <c r="BN11" s="384"/>
+      <c r="BO11" s="384"/>
+      <c r="BP11" s="384"/>
+      <c r="BQ11" s="384"/>
+      <c r="BR11" s="384"/>
+      <c r="BS11" s="384"/>
+      <c r="BT11" s="384"/>
+      <c r="BU11" s="394"/>
       <c r="BV11" s="114"/>
-      <c r="BW11" s="414"/>
+      <c r="BW11" s="413"/>
       <c r="BX11" s="72" t="s">
         <v>91</v>
       </c>
@@ -15904,9 +15904,9 @@
       <c r="CA11" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="CB11" s="406"/>
-      <c r="CC11" s="406"/>
-      <c r="CD11" s="406"/>
+      <c r="CB11" s="405"/>
+      <c r="CC11" s="405"/>
+      <c r="CD11" s="405"/>
       <c r="CE11" s="11"/>
       <c r="CF11" s="31"/>
       <c r="CH11" s="27"/>
@@ -18618,87 +18618,87 @@
       <c r="CD2" s="132"/>
     </row>
     <row r="3" spans="1:87" s="134" customFormat="1" ht="11" outlineLevel="1">
-      <c r="A3" s="416"/>
-      <c r="B3" s="404"/>
-      <c r="C3" s="404"/>
-      <c r="D3" s="404"/>
-      <c r="E3" s="404"/>
-      <c r="F3" s="404"/>
-      <c r="G3" s="404"/>
-      <c r="H3" s="404"/>
-      <c r="I3" s="404"/>
-      <c r="J3" s="404"/>
-      <c r="K3" s="404"/>
-      <c r="L3" s="404"/>
-      <c r="M3" s="404"/>
-      <c r="N3" s="404"/>
-      <c r="O3" s="404"/>
-      <c r="P3" s="404"/>
-      <c r="Q3" s="404"/>
-      <c r="R3" s="404"/>
-      <c r="S3" s="404"/>
-      <c r="T3" s="404"/>
-      <c r="U3" s="404"/>
-      <c r="V3" s="404"/>
-      <c r="W3" s="404"/>
-      <c r="X3" s="404"/>
-      <c r="Y3" s="404"/>
-      <c r="Z3" s="404"/>
-      <c r="AA3" s="404"/>
-      <c r="AB3" s="404"/>
-      <c r="AC3" s="404"/>
-      <c r="AD3" s="404"/>
-      <c r="AE3" s="404"/>
-      <c r="AF3" s="404"/>
-      <c r="AG3" s="404"/>
-      <c r="AH3" s="404"/>
-      <c r="AI3" s="404"/>
-      <c r="AJ3" s="404"/>
-      <c r="AK3" s="404"/>
-      <c r="AL3" s="404"/>
-      <c r="AM3" s="404"/>
-      <c r="AN3" s="404"/>
-      <c r="AO3" s="404"/>
-      <c r="AP3" s="404"/>
-      <c r="AQ3" s="404"/>
-      <c r="AR3" s="404"/>
-      <c r="AS3" s="404"/>
-      <c r="AT3" s="404"/>
-      <c r="AU3" s="404"/>
-      <c r="AV3" s="404"/>
-      <c r="AW3" s="404"/>
-      <c r="AX3" s="404"/>
-      <c r="AY3" s="404"/>
-      <c r="AZ3" s="404"/>
-      <c r="BA3" s="404"/>
-      <c r="BB3" s="404"/>
-      <c r="BC3" s="404"/>
-      <c r="BD3" s="404"/>
-      <c r="BE3" s="404"/>
-      <c r="BF3" s="404"/>
-      <c r="BG3" s="404"/>
-      <c r="BH3" s="404"/>
-      <c r="BI3" s="404"/>
-      <c r="BJ3" s="404"/>
-      <c r="BK3" s="404"/>
-      <c r="BL3" s="404"/>
-      <c r="BM3" s="404"/>
-      <c r="BN3" s="404"/>
-      <c r="BO3" s="404"/>
-      <c r="BP3" s="404"/>
-      <c r="BQ3" s="404"/>
-      <c r="BR3" s="404"/>
-      <c r="BS3" s="404"/>
-      <c r="BT3" s="404"/>
-      <c r="BU3" s="404"/>
-      <c r="BW3" s="403" t="s">
+      <c r="A3" s="415"/>
+      <c r="B3" s="403"/>
+      <c r="C3" s="403"/>
+      <c r="D3" s="403"/>
+      <c r="E3" s="403"/>
+      <c r="F3" s="403"/>
+      <c r="G3" s="403"/>
+      <c r="H3" s="403"/>
+      <c r="I3" s="403"/>
+      <c r="J3" s="403"/>
+      <c r="K3" s="403"/>
+      <c r="L3" s="403"/>
+      <c r="M3" s="403"/>
+      <c r="N3" s="403"/>
+      <c r="O3" s="403"/>
+      <c r="P3" s="403"/>
+      <c r="Q3" s="403"/>
+      <c r="R3" s="403"/>
+      <c r="S3" s="403"/>
+      <c r="T3" s="403"/>
+      <c r="U3" s="403"/>
+      <c r="V3" s="403"/>
+      <c r="W3" s="403"/>
+      <c r="X3" s="403"/>
+      <c r="Y3" s="403"/>
+      <c r="Z3" s="403"/>
+      <c r="AA3" s="403"/>
+      <c r="AB3" s="403"/>
+      <c r="AC3" s="403"/>
+      <c r="AD3" s="403"/>
+      <c r="AE3" s="403"/>
+      <c r="AF3" s="403"/>
+      <c r="AG3" s="403"/>
+      <c r="AH3" s="403"/>
+      <c r="AI3" s="403"/>
+      <c r="AJ3" s="403"/>
+      <c r="AK3" s="403"/>
+      <c r="AL3" s="403"/>
+      <c r="AM3" s="403"/>
+      <c r="AN3" s="403"/>
+      <c r="AO3" s="403"/>
+      <c r="AP3" s="403"/>
+      <c r="AQ3" s="403"/>
+      <c r="AR3" s="403"/>
+      <c r="AS3" s="403"/>
+      <c r="AT3" s="403"/>
+      <c r="AU3" s="403"/>
+      <c r="AV3" s="403"/>
+      <c r="AW3" s="403"/>
+      <c r="AX3" s="403"/>
+      <c r="AY3" s="403"/>
+      <c r="AZ3" s="403"/>
+      <c r="BA3" s="403"/>
+      <c r="BB3" s="403"/>
+      <c r="BC3" s="403"/>
+      <c r="BD3" s="403"/>
+      <c r="BE3" s="403"/>
+      <c r="BF3" s="403"/>
+      <c r="BG3" s="403"/>
+      <c r="BH3" s="403"/>
+      <c r="BI3" s="403"/>
+      <c r="BJ3" s="403"/>
+      <c r="BK3" s="403"/>
+      <c r="BL3" s="403"/>
+      <c r="BM3" s="403"/>
+      <c r="BN3" s="403"/>
+      <c r="BO3" s="403"/>
+      <c r="BP3" s="403"/>
+      <c r="BQ3" s="403"/>
+      <c r="BR3" s="403"/>
+      <c r="BS3" s="403"/>
+      <c r="BT3" s="403"/>
+      <c r="BU3" s="403"/>
+      <c r="BW3" s="402" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="404"/>
-      <c r="BY3" s="404"/>
-      <c r="BZ3" s="404"/>
-      <c r="CA3" s="404"/>
-      <c r="CB3" s="404"/>
+      <c r="BX3" s="403"/>
+      <c r="BY3" s="403"/>
+      <c r="BZ3" s="403"/>
+      <c r="CA3" s="403"/>
+      <c r="CB3" s="403"/>
       <c r="CC3" s="133"/>
       <c r="CD3" s="133"/>
       <c r="CE3" s="134" t="s">
@@ -18781,366 +18781,366 @@
       <c r="BS4" s="135"/>
       <c r="BT4" s="135"/>
       <c r="BU4" s="135"/>
-      <c r="BW4" s="404"/>
-      <c r="BX4" s="404"/>
-      <c r="BY4" s="404"/>
-      <c r="BZ4" s="404"/>
-      <c r="CA4" s="404"/>
-      <c r="CB4" s="404"/>
+      <c r="BW4" s="403"/>
+      <c r="BX4" s="403"/>
+      <c r="BY4" s="403"/>
+      <c r="BZ4" s="403"/>
+      <c r="CA4" s="403"/>
+      <c r="CB4" s="403"/>
       <c r="CC4" s="133"/>
       <c r="CD4" s="133"/>
     </row>
     <row r="5" spans="1:87" s="136" customFormat="1">
-      <c r="A5" s="392" t="s">
+      <c r="A5" s="391" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="402" t="s">
+      <c r="B5" s="401" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="390" t="s">
+      <c r="C5" s="389" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="398" t="s">
+      <c r="D5" s="397" t="s">
         <v>141</v>
       </c>
-      <c r="E5" s="398" t="s">
+      <c r="E5" s="397" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="427" t="s">
+      <c r="F5" s="426" t="s">
         <v>142</v>
       </c>
-      <c r="G5" s="390" t="s">
+      <c r="G5" s="389" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="346" t="s">
+      <c r="H5" s="345" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="346" t="s">
+      <c r="I5" s="345" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="390" t="s">
+      <c r="J5" s="389" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="396" t="s">
+      <c r="K5" s="395" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="387"/>
-      <c r="M5" s="387"/>
-      <c r="N5" s="387"/>
-      <c r="O5" s="387"/>
-      <c r="P5" s="387"/>
-      <c r="Q5" s="387"/>
-      <c r="R5" s="387"/>
-      <c r="S5" s="387"/>
-      <c r="T5" s="387"/>
-      <c r="U5" s="387"/>
-      <c r="V5" s="387"/>
-      <c r="W5" s="387"/>
-      <c r="X5" s="387"/>
-      <c r="Y5" s="390" t="s">
+      <c r="L5" s="386"/>
+      <c r="M5" s="386"/>
+      <c r="N5" s="386"/>
+      <c r="O5" s="386"/>
+      <c r="P5" s="386"/>
+      <c r="Q5" s="386"/>
+      <c r="R5" s="386"/>
+      <c r="S5" s="386"/>
+      <c r="T5" s="386"/>
+      <c r="U5" s="386"/>
+      <c r="V5" s="386"/>
+      <c r="W5" s="386"/>
+      <c r="X5" s="386"/>
+      <c r="Y5" s="389" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="387"/>
-      <c r="AA5" s="387"/>
-      <c r="AB5" s="387"/>
-      <c r="AC5" s="387"/>
-      <c r="AD5" s="387"/>
-      <c r="AE5" s="387"/>
-      <c r="AF5" s="387"/>
-      <c r="AG5" s="387"/>
-      <c r="AH5" s="387"/>
-      <c r="AI5" s="387"/>
-      <c r="AJ5" s="387"/>
-      <c r="AK5" s="387"/>
-      <c r="AL5" s="387"/>
-      <c r="AM5" s="387"/>
-      <c r="AN5" s="387"/>
-      <c r="AO5" s="388"/>
-      <c r="AP5" s="390" t="s">
+      <c r="Z5" s="386"/>
+      <c r="AA5" s="386"/>
+      <c r="AB5" s="386"/>
+      <c r="AC5" s="386"/>
+      <c r="AD5" s="386"/>
+      <c r="AE5" s="386"/>
+      <c r="AF5" s="386"/>
+      <c r="AG5" s="386"/>
+      <c r="AH5" s="386"/>
+      <c r="AI5" s="386"/>
+      <c r="AJ5" s="386"/>
+      <c r="AK5" s="386"/>
+      <c r="AL5" s="386"/>
+      <c r="AM5" s="386"/>
+      <c r="AN5" s="386"/>
+      <c r="AO5" s="387"/>
+      <c r="AP5" s="389" t="s">
         <v>16</v>
       </c>
-      <c r="AQ5" s="390" t="s">
+      <c r="AQ5" s="389" t="s">
         <v>17</v>
       </c>
-      <c r="AR5" s="390" t="s">
+      <c r="AR5" s="389" t="s">
         <v>18</v>
       </c>
-      <c r="AS5" s="390" t="s">
+      <c r="AS5" s="389" t="s">
         <v>19</v>
       </c>
-      <c r="AT5" s="390" t="s">
+      <c r="AT5" s="389" t="s">
         <v>20</v>
       </c>
-      <c r="AU5" s="390" t="s">
+      <c r="AU5" s="389" t="s">
         <v>21</v>
       </c>
-      <c r="AV5" s="390" t="s">
+      <c r="AV5" s="389" t="s">
         <v>22</v>
       </c>
-      <c r="AW5" s="390" t="s">
+      <c r="AW5" s="389" t="s">
         <v>23</v>
       </c>
-      <c r="AX5" s="390" t="s">
+      <c r="AX5" s="389" t="s">
         <v>24</v>
       </c>
-      <c r="AY5" s="386" t="s">
+      <c r="AY5" s="385" t="s">
         <v>25</v>
       </c>
-      <c r="AZ5" s="387"/>
-      <c r="BA5" s="387"/>
-      <c r="BB5" s="387"/>
-      <c r="BC5" s="387"/>
-      <c r="BD5" s="387"/>
-      <c r="BE5" s="387"/>
-      <c r="BF5" s="387"/>
-      <c r="BG5" s="387"/>
-      <c r="BH5" s="387"/>
-      <c r="BI5" s="387"/>
-      <c r="BJ5" s="387"/>
-      <c r="BK5" s="387"/>
-      <c r="BL5" s="387"/>
-      <c r="BM5" s="387"/>
-      <c r="BN5" s="387"/>
-      <c r="BO5" s="387"/>
-      <c r="BP5" s="388"/>
-      <c r="BQ5" s="407" t="s">
+      <c r="AZ5" s="386"/>
+      <c r="BA5" s="386"/>
+      <c r="BB5" s="386"/>
+      <c r="BC5" s="386"/>
+      <c r="BD5" s="386"/>
+      <c r="BE5" s="386"/>
+      <c r="BF5" s="386"/>
+      <c r="BG5" s="386"/>
+      <c r="BH5" s="386"/>
+      <c r="BI5" s="386"/>
+      <c r="BJ5" s="386"/>
+      <c r="BK5" s="386"/>
+      <c r="BL5" s="386"/>
+      <c r="BM5" s="386"/>
+      <c r="BN5" s="386"/>
+      <c r="BO5" s="386"/>
+      <c r="BP5" s="387"/>
+      <c r="BQ5" s="406" t="s">
         <v>26</v>
       </c>
-      <c r="BR5" s="400"/>
-      <c r="BS5" s="386" t="s">
+      <c r="BR5" s="399"/>
+      <c r="BS5" s="385" t="s">
         <v>143</v>
       </c>
-      <c r="BT5" s="386" t="s">
+      <c r="BT5" s="385" t="s">
         <v>27</v>
       </c>
-      <c r="BU5" s="418" t="s">
+      <c r="BU5" s="417" t="s">
         <v>28</v>
       </c>
-      <c r="BW5" s="419" t="s">
+      <c r="BW5" s="418" t="s">
         <v>29</v>
       </c>
-      <c r="BX5" s="408" t="s">
+      <c r="BX5" s="407" t="s">
         <v>30</v>
       </c>
-      <c r="BY5" s="409"/>
-      <c r="BZ5" s="409"/>
-      <c r="CA5" s="400"/>
-      <c r="CB5" s="420" t="s">
+      <c r="BY5" s="408"/>
+      <c r="BZ5" s="408"/>
+      <c r="CA5" s="399"/>
+      <c r="CB5" s="419" t="s">
         <v>31</v>
       </c>
-      <c r="CC5" s="405" t="s">
+      <c r="CC5" s="404" t="s">
         <v>32</v>
       </c>
-      <c r="CD5" s="405" t="s">
+      <c r="CD5" s="404" t="s">
         <v>33</v>
       </c>
       <c r="CH5" s="137"/>
       <c r="CI5" s="138"/>
     </row>
     <row r="6" spans="1:87" s="136" customFormat="1">
-      <c r="A6" s="384"/>
-      <c r="B6" s="384"/>
-      <c r="C6" s="384"/>
-      <c r="D6" s="384"/>
-      <c r="E6" s="384"/>
-      <c r="F6" s="384"/>
-      <c r="G6" s="384"/>
-      <c r="H6" s="384"/>
-      <c r="I6" s="384"/>
-      <c r="J6" s="384"/>
-      <c r="K6" s="391" t="s">
+      <c r="A6" s="383"/>
+      <c r="B6" s="383"/>
+      <c r="C6" s="383"/>
+      <c r="D6" s="383"/>
+      <c r="E6" s="383"/>
+      <c r="F6" s="383"/>
+      <c r="G6" s="383"/>
+      <c r="H6" s="383"/>
+      <c r="I6" s="383"/>
+      <c r="J6" s="383"/>
+      <c r="K6" s="390" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="391" t="s">
+      <c r="L6" s="390" t="s">
         <v>35</v>
       </c>
-      <c r="M6" s="391" t="s">
+      <c r="M6" s="390" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="391" t="s">
+      <c r="N6" s="390" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="391" t="s">
+      <c r="O6" s="390" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="391" t="s">
+      <c r="P6" s="390" t="s">
         <v>39</v>
       </c>
-      <c r="Q6" s="391" t="s">
+      <c r="Q6" s="390" t="s">
         <v>40</v>
       </c>
-      <c r="R6" s="391" t="s">
+      <c r="R6" s="390" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="391" t="s">
+      <c r="S6" s="390" t="s">
         <v>42</v>
       </c>
-      <c r="T6" s="391" t="s">
+      <c r="T6" s="390" t="s">
         <v>43</v>
       </c>
-      <c r="U6" s="391" t="s">
+      <c r="U6" s="390" t="s">
         <v>44</v>
       </c>
-      <c r="V6" s="399" t="s">
+      <c r="V6" s="398" t="s">
         <v>45</v>
       </c>
-      <c r="W6" s="400"/>
-      <c r="X6" s="391" t="s">
+      <c r="W6" s="399"/>
+      <c r="X6" s="390" t="s">
         <v>46</v>
       </c>
-      <c r="Y6" s="390" t="s">
+      <c r="Y6" s="389" t="s">
         <v>47</v>
       </c>
-      <c r="Z6" s="390" t="s">
+      <c r="Z6" s="389" t="s">
         <v>48</v>
       </c>
-      <c r="AA6" s="390" t="s">
+      <c r="AA6" s="389" t="s">
         <v>49</v>
       </c>
-      <c r="AB6" s="390" t="s">
+      <c r="AB6" s="389" t="s">
         <v>50</v>
       </c>
-      <c r="AC6" s="346" t="s">
+      <c r="AC6" s="345" t="s">
         <v>51</v>
       </c>
-      <c r="AD6" s="346" t="s">
+      <c r="AD6" s="345" t="s">
         <v>144</v>
       </c>
-      <c r="AE6" s="346" t="s">
+      <c r="AE6" s="345" t="s">
         <v>53</v>
       </c>
-      <c r="AF6" s="346" t="s">
+      <c r="AF6" s="345" t="s">
         <v>54</v>
       </c>
-      <c r="AG6" s="390" t="s">
+      <c r="AG6" s="389" t="s">
         <v>55</v>
       </c>
-      <c r="AH6" s="346" t="s">
+      <c r="AH6" s="345" t="s">
         <v>56</v>
       </c>
-      <c r="AI6" s="346" t="s">
+      <c r="AI6" s="345" t="s">
         <v>57</v>
       </c>
-      <c r="AJ6" s="390" t="s">
+      <c r="AJ6" s="389" t="s">
         <v>58</v>
       </c>
-      <c r="AK6" s="393" t="s">
+      <c r="AK6" s="392" t="s">
         <v>59</v>
       </c>
-      <c r="AL6" s="390" t="s">
+      <c r="AL6" s="389" t="s">
         <v>60</v>
       </c>
-      <c r="AM6" s="390" t="s">
+      <c r="AM6" s="389" t="s">
         <v>61</v>
       </c>
-      <c r="AN6" s="397" t="s">
+      <c r="AN6" s="396" t="s">
         <v>62</v>
       </c>
-      <c r="AO6" s="390" t="s">
+      <c r="AO6" s="389" t="s">
         <v>63</v>
       </c>
-      <c r="AP6" s="384"/>
-      <c r="AQ6" s="384"/>
-      <c r="AR6" s="384"/>
-      <c r="AS6" s="384"/>
-      <c r="AT6" s="384"/>
-      <c r="AU6" s="384"/>
-      <c r="AV6" s="384"/>
-      <c r="AW6" s="384"/>
-      <c r="AX6" s="384"/>
-      <c r="AY6" s="386" t="s">
+      <c r="AP6" s="383"/>
+      <c r="AQ6" s="383"/>
+      <c r="AR6" s="383"/>
+      <c r="AS6" s="383"/>
+      <c r="AT6" s="383"/>
+      <c r="AU6" s="383"/>
+      <c r="AV6" s="383"/>
+      <c r="AW6" s="383"/>
+      <c r="AX6" s="383"/>
+      <c r="AY6" s="385" t="s">
         <v>25</v>
       </c>
-      <c r="AZ6" s="387"/>
-      <c r="BA6" s="387"/>
-      <c r="BB6" s="387"/>
-      <c r="BC6" s="387"/>
-      <c r="BD6" s="387"/>
-      <c r="BE6" s="387"/>
-      <c r="BF6" s="387"/>
-      <c r="BG6" s="387"/>
-      <c r="BH6" s="387"/>
-      <c r="BI6" s="387"/>
-      <c r="BJ6" s="388"/>
-      <c r="BK6" s="386" t="s">
+      <c r="AZ6" s="386"/>
+      <c r="BA6" s="386"/>
+      <c r="BB6" s="386"/>
+      <c r="BC6" s="386"/>
+      <c r="BD6" s="386"/>
+      <c r="BE6" s="386"/>
+      <c r="BF6" s="386"/>
+      <c r="BG6" s="386"/>
+      <c r="BH6" s="386"/>
+      <c r="BI6" s="386"/>
+      <c r="BJ6" s="387"/>
+      <c r="BK6" s="385" t="s">
         <v>64</v>
       </c>
-      <c r="BL6" s="387"/>
-      <c r="BM6" s="387"/>
-      <c r="BN6" s="387"/>
-      <c r="BO6" s="387"/>
-      <c r="BP6" s="388"/>
-      <c r="BQ6" s="383" t="s">
+      <c r="BL6" s="386"/>
+      <c r="BM6" s="386"/>
+      <c r="BN6" s="386"/>
+      <c r="BO6" s="386"/>
+      <c r="BP6" s="387"/>
+      <c r="BQ6" s="382" t="s">
         <v>65</v>
       </c>
-      <c r="BR6" s="383" t="s">
+      <c r="BR6" s="382" t="s">
         <v>66</v>
       </c>
-      <c r="BS6" s="384"/>
-      <c r="BT6" s="384"/>
-      <c r="BU6" s="394"/>
-      <c r="BW6" s="411"/>
-      <c r="BX6" s="394"/>
-      <c r="BY6" s="410"/>
-      <c r="BZ6" s="410"/>
-      <c r="CA6" s="411"/>
-      <c r="CB6" s="384"/>
-      <c r="CC6" s="384"/>
-      <c r="CD6" s="384"/>
+      <c r="BS6" s="383"/>
+      <c r="BT6" s="383"/>
+      <c r="BU6" s="393"/>
+      <c r="BW6" s="410"/>
+      <c r="BX6" s="393"/>
+      <c r="BY6" s="409"/>
+      <c r="BZ6" s="409"/>
+      <c r="CA6" s="410"/>
+      <c r="CB6" s="383"/>
+      <c r="CC6" s="383"/>
+      <c r="CD6" s="383"/>
       <c r="CH6" s="137"/>
       <c r="CI6" s="138"/>
     </row>
     <row r="7" spans="1:87" s="136" customFormat="1" ht="12">
-      <c r="A7" s="384"/>
-      <c r="B7" s="384"/>
-      <c r="C7" s="384"/>
-      <c r="D7" s="384"/>
-      <c r="E7" s="384"/>
-      <c r="F7" s="384"/>
-      <c r="G7" s="384"/>
-      <c r="H7" s="384"/>
-      <c r="I7" s="384"/>
-      <c r="J7" s="384"/>
-      <c r="K7" s="384"/>
-      <c r="L7" s="384"/>
-      <c r="M7" s="384"/>
-      <c r="N7" s="384"/>
-      <c r="O7" s="384"/>
-      <c r="P7" s="384"/>
-      <c r="Q7" s="384"/>
-      <c r="R7" s="384"/>
-      <c r="S7" s="384"/>
-      <c r="T7" s="384"/>
-      <c r="U7" s="384"/>
-      <c r="V7" s="395"/>
-      <c r="W7" s="401"/>
-      <c r="X7" s="384"/>
-      <c r="Y7" s="384"/>
-      <c r="Z7" s="384"/>
-      <c r="AA7" s="384"/>
-      <c r="AB7" s="384"/>
-      <c r="AC7" s="384"/>
-      <c r="AD7" s="384"/>
-      <c r="AE7" s="384"/>
-      <c r="AF7" s="384"/>
-      <c r="AG7" s="384"/>
-      <c r="AH7" s="384"/>
-      <c r="AI7" s="384"/>
-      <c r="AJ7" s="384"/>
-      <c r="AK7" s="394"/>
-      <c r="AL7" s="384"/>
-      <c r="AM7" s="384"/>
-      <c r="AN7" s="384"/>
-      <c r="AO7" s="384"/>
-      <c r="AP7" s="384"/>
-      <c r="AQ7" s="384"/>
-      <c r="AR7" s="384"/>
-      <c r="AS7" s="384"/>
-      <c r="AT7" s="384"/>
-      <c r="AU7" s="384"/>
-      <c r="AV7" s="384"/>
-      <c r="AW7" s="384"/>
-      <c r="AX7" s="384"/>
+      <c r="A7" s="383"/>
+      <c r="B7" s="383"/>
+      <c r="C7" s="383"/>
+      <c r="D7" s="383"/>
+      <c r="E7" s="383"/>
+      <c r="F7" s="383"/>
+      <c r="G7" s="383"/>
+      <c r="H7" s="383"/>
+      <c r="I7" s="383"/>
+      <c r="J7" s="383"/>
+      <c r="K7" s="383"/>
+      <c r="L7" s="383"/>
+      <c r="M7" s="383"/>
+      <c r="N7" s="383"/>
+      <c r="O7" s="383"/>
+      <c r="P7" s="383"/>
+      <c r="Q7" s="383"/>
+      <c r="R7" s="383"/>
+      <c r="S7" s="383"/>
+      <c r="T7" s="383"/>
+      <c r="U7" s="383"/>
+      <c r="V7" s="394"/>
+      <c r="W7" s="400"/>
+      <c r="X7" s="383"/>
+      <c r="Y7" s="383"/>
+      <c r="Z7" s="383"/>
+      <c r="AA7" s="383"/>
+      <c r="AB7" s="383"/>
+      <c r="AC7" s="383"/>
+      <c r="AD7" s="383"/>
+      <c r="AE7" s="383"/>
+      <c r="AF7" s="383"/>
+      <c r="AG7" s="383"/>
+      <c r="AH7" s="383"/>
+      <c r="AI7" s="383"/>
+      <c r="AJ7" s="383"/>
+      <c r="AK7" s="393"/>
+      <c r="AL7" s="383"/>
+      <c r="AM7" s="383"/>
+      <c r="AN7" s="383"/>
+      <c r="AO7" s="383"/>
+      <c r="AP7" s="383"/>
+      <c r="AQ7" s="383"/>
+      <c r="AR7" s="383"/>
+      <c r="AS7" s="383"/>
+      <c r="AT7" s="383"/>
+      <c r="AU7" s="383"/>
+      <c r="AV7" s="383"/>
+      <c r="AW7" s="383"/>
+      <c r="AX7" s="383"/>
       <c r="AY7" s="101" t="s">
         <v>67</v>
       </c>
@@ -19150,122 +19150,122 @@
       <c r="BA7" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="BB7" s="386" t="s">
+      <c r="BB7" s="385" t="s">
         <v>70</v>
       </c>
-      <c r="BC7" s="389" t="s">
+      <c r="BC7" s="388" t="s">
         <v>71</v>
       </c>
-      <c r="BD7" s="389" t="s">
+      <c r="BD7" s="388" t="s">
         <v>72</v>
       </c>
-      <c r="BE7" s="389" t="s">
+      <c r="BE7" s="388" t="s">
         <v>145</v>
       </c>
-      <c r="BF7" s="389" t="s">
+      <c r="BF7" s="388" t="s">
         <v>74</v>
       </c>
-      <c r="BG7" s="389" t="s">
+      <c r="BG7" s="388" t="s">
         <v>75</v>
       </c>
-      <c r="BH7" s="389" t="s">
+      <c r="BH7" s="388" t="s">
         <v>76</v>
       </c>
-      <c r="BI7" s="389" t="s">
+      <c r="BI7" s="388" t="s">
         <v>79</v>
       </c>
-      <c r="BJ7" s="417" t="s">
+      <c r="BJ7" s="416" t="s">
         <v>80</v>
       </c>
-      <c r="BK7" s="389" t="s">
+      <c r="BK7" s="388" t="s">
         <v>81</v>
       </c>
-      <c r="BL7" s="386" t="s">
+      <c r="BL7" s="385" t="s">
         <v>82</v>
       </c>
-      <c r="BM7" s="389" t="s">
+      <c r="BM7" s="388" t="s">
         <v>83</v>
       </c>
-      <c r="BN7" s="386" t="s">
+      <c r="BN7" s="385" t="s">
         <v>84</v>
       </c>
-      <c r="BO7" s="386" t="s">
+      <c r="BO7" s="385" t="s">
         <v>146</v>
       </c>
-      <c r="BP7" s="386" t="s">
+      <c r="BP7" s="385" t="s">
         <v>85</v>
       </c>
-      <c r="BQ7" s="384"/>
-      <c r="BR7" s="384"/>
-      <c r="BS7" s="384"/>
-      <c r="BT7" s="384"/>
-      <c r="BU7" s="394"/>
-      <c r="BW7" s="411"/>
-      <c r="BX7" s="412"/>
-      <c r="BY7" s="413"/>
-      <c r="BZ7" s="413"/>
-      <c r="CA7" s="414"/>
-      <c r="CB7" s="384"/>
-      <c r="CC7" s="384"/>
-      <c r="CD7" s="384"/>
+      <c r="BQ7" s="383"/>
+      <c r="BR7" s="383"/>
+      <c r="BS7" s="383"/>
+      <c r="BT7" s="383"/>
+      <c r="BU7" s="393"/>
+      <c r="BW7" s="410"/>
+      <c r="BX7" s="411"/>
+      <c r="BY7" s="412"/>
+      <c r="BZ7" s="412"/>
+      <c r="CA7" s="413"/>
+      <c r="CB7" s="383"/>
+      <c r="CC7" s="383"/>
+      <c r="CD7" s="383"/>
       <c r="CH7" s="137"/>
       <c r="CI7" s="138"/>
     </row>
     <row r="8" spans="1:87" s="136" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A8" s="385"/>
-      <c r="B8" s="385"/>
-      <c r="C8" s="385"/>
-      <c r="D8" s="385"/>
-      <c r="E8" s="385"/>
-      <c r="F8" s="385"/>
-      <c r="G8" s="385"/>
-      <c r="H8" s="385"/>
-      <c r="I8" s="385"/>
-      <c r="J8" s="385"/>
-      <c r="K8" s="385"/>
-      <c r="L8" s="385"/>
-      <c r="M8" s="385"/>
-      <c r="N8" s="385"/>
-      <c r="O8" s="385"/>
-      <c r="P8" s="385"/>
-      <c r="Q8" s="385"/>
-      <c r="R8" s="385"/>
-      <c r="S8" s="385"/>
-      <c r="T8" s="385"/>
-      <c r="U8" s="385"/>
+      <c r="A8" s="384"/>
+      <c r="B8" s="384"/>
+      <c r="C8" s="384"/>
+      <c r="D8" s="384"/>
+      <c r="E8" s="384"/>
+      <c r="F8" s="384"/>
+      <c r="G8" s="384"/>
+      <c r="H8" s="384"/>
+      <c r="I8" s="384"/>
+      <c r="J8" s="384"/>
+      <c r="K8" s="384"/>
+      <c r="L8" s="384"/>
+      <c r="M8" s="384"/>
+      <c r="N8" s="384"/>
+      <c r="O8" s="384"/>
+      <c r="P8" s="384"/>
+      <c r="Q8" s="384"/>
+      <c r="R8" s="384"/>
+      <c r="S8" s="384"/>
+      <c r="T8" s="384"/>
+      <c r="U8" s="384"/>
       <c r="V8" s="140" t="s">
         <v>86</v>
       </c>
       <c r="W8" s="140" t="s">
         <v>87</v>
       </c>
-      <c r="X8" s="385"/>
-      <c r="Y8" s="385"/>
-      <c r="Z8" s="385"/>
-      <c r="AA8" s="385"/>
-      <c r="AB8" s="385"/>
-      <c r="AC8" s="385"/>
-      <c r="AD8" s="385"/>
-      <c r="AE8" s="385"/>
-      <c r="AF8" s="385"/>
-      <c r="AG8" s="385"/>
-      <c r="AH8" s="385"/>
-      <c r="AI8" s="385"/>
-      <c r="AJ8" s="385"/>
-      <c r="AK8" s="395"/>
-      <c r="AL8" s="385"/>
-      <c r="AM8" s="385"/>
-      <c r="AN8" s="385"/>
-      <c r="AO8" s="385"/>
-      <c r="AP8" s="385"/>
-      <c r="AQ8" s="385"/>
-      <c r="AR8" s="385"/>
-      <c r="AS8" s="385"/>
-      <c r="AT8" s="385"/>
-      <c r="AU8" s="385"/>
-      <c r="AV8" s="385"/>
-      <c r="AW8" s="385"/>
-      <c r="AX8" s="385"/>
+      <c r="X8" s="384"/>
+      <c r="Y8" s="384"/>
+      <c r="Z8" s="384"/>
+      <c r="AA8" s="384"/>
+      <c r="AB8" s="384"/>
+      <c r="AC8" s="384"/>
+      <c r="AD8" s="384"/>
+      <c r="AE8" s="384"/>
+      <c r="AF8" s="384"/>
+      <c r="AG8" s="384"/>
+      <c r="AH8" s="384"/>
+      <c r="AI8" s="384"/>
+      <c r="AJ8" s="384"/>
+      <c r="AK8" s="394"/>
+      <c r="AL8" s="384"/>
+      <c r="AM8" s="384"/>
+      <c r="AN8" s="384"/>
+      <c r="AO8" s="384"/>
+      <c r="AP8" s="384"/>
+      <c r="AQ8" s="384"/>
+      <c r="AR8" s="384"/>
+      <c r="AS8" s="384"/>
+      <c r="AT8" s="384"/>
+      <c r="AU8" s="384"/>
+      <c r="AV8" s="384"/>
+      <c r="AW8" s="384"/>
+      <c r="AX8" s="384"/>
       <c r="AY8" s="102" t="s">
         <v>88</v>
       </c>
@@ -19275,27 +19275,27 @@
       <c r="BA8" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="BB8" s="385"/>
-      <c r="BC8" s="385"/>
-      <c r="BD8" s="385"/>
-      <c r="BE8" s="385"/>
-      <c r="BF8" s="385"/>
-      <c r="BG8" s="385"/>
-      <c r="BH8" s="385"/>
-      <c r="BI8" s="385"/>
-      <c r="BJ8" s="385"/>
-      <c r="BK8" s="385"/>
-      <c r="BL8" s="385"/>
-      <c r="BM8" s="385"/>
-      <c r="BN8" s="385"/>
-      <c r="BO8" s="385"/>
-      <c r="BP8" s="385"/>
-      <c r="BQ8" s="385"/>
-      <c r="BR8" s="385"/>
-      <c r="BS8" s="385"/>
-      <c r="BT8" s="385"/>
-      <c r="BU8" s="395"/>
-      <c r="BW8" s="414"/>
+      <c r="BB8" s="384"/>
+      <c r="BC8" s="384"/>
+      <c r="BD8" s="384"/>
+      <c r="BE8" s="384"/>
+      <c r="BF8" s="384"/>
+      <c r="BG8" s="384"/>
+      <c r="BH8" s="384"/>
+      <c r="BI8" s="384"/>
+      <c r="BJ8" s="384"/>
+      <c r="BK8" s="384"/>
+      <c r="BL8" s="384"/>
+      <c r="BM8" s="384"/>
+      <c r="BN8" s="384"/>
+      <c r="BO8" s="384"/>
+      <c r="BP8" s="384"/>
+      <c r="BQ8" s="384"/>
+      <c r="BR8" s="384"/>
+      <c r="BS8" s="384"/>
+      <c r="BT8" s="384"/>
+      <c r="BU8" s="394"/>
+      <c r="BW8" s="413"/>
       <c r="BX8" s="72" t="s">
         <v>91</v>
       </c>
@@ -19308,9 +19308,9 @@
       <c r="CA8" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="CB8" s="406"/>
-      <c r="CC8" s="406"/>
-      <c r="CD8" s="406"/>
+      <c r="CB8" s="405"/>
+      <c r="CC8" s="405"/>
+      <c r="CD8" s="405"/>
       <c r="CF8" s="141"/>
       <c r="CH8" s="137"/>
       <c r="CI8" s="138"/>

</xml_diff>